<commit_message>
Communications: 12 not-yet-available SMS rewritten and added (LAN, expiry, discard, post-pledge, lien removal, withdrawal rejected); Excel export script and refreshed export
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -10,7 +10,7 @@
     <sheet name="LAMF Communications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LAMF Communications'!$A$1:$K$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LAMF Communications'!$A$1:$K$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,13 +103,13 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -723,57 +723,57 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Pledging of Mutual Fund</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>After the mutual fund units are successfully pledged on the “Pledging of Mutual Fund” page (Pledge Securities → MF Central OTP → “Successfully pledged!”)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>LAN Generated</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>When the customer clicks Continue on the Loan Application Summary page and the Loan Account Number (LAN) is generated successfully</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is {#alphanumeric#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -783,12 +783,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Lien Marking Failed</t>
+          <t>Pre-Pledge Application Expiry Reminder</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
+          <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -833,112 +833,112 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Sanction Letter</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>After the Sanction Letter is generated successfully (customer clicks “Sign Agreement” on the “Agreement and E-Mandate” page and the Sanction Letter is generated)</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Pledge Application Discarded</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Loan Agreement e-Sign</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>After the customer signs the loan agreement successfully (e-Sign at Digio – Aadhaar / VID + OTP → “Signed Successfully”)</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Customer-Initiated Discard</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -948,12 +948,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>LAMF Application Submit</t>
+          <t>Pledging of Mutual Fund</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
+          <t>After the mutual fund units are successfully pledged on the “Pledging of Mutual Fund” page (Pledge Securities → MF Central OTP → “Successfully pledged!”)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -998,57 +998,57 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Loan Lodgement Approval</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>After the application is submitted, the OPS team approves in the backend LMS, back to back: first the Loan Account Opening approval, then the Loan Lodgement approval. This SMS is triggered when the Loan Lodgement is approved</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alp#}, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Lien Marking Failed</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -1058,17 +1058,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Loan Account Opening / Loan Lodgement Rejection</t>
+          <t>Post-Pledge Journey Incomplete</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection, with a payment link for the charges the customer has to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
+          <t>Lien marking is successful, then the customer is inactive for the configured period</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>LMS</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -1108,332 +1108,332 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Post-Pledge Application Expiry Reminder</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Application Expired – Lien Marked</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>The application reaches Day 31 without submission and the lien is still marked</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Loan Disbursed</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Lien Removal Request Received</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SCCL receives and records the customer’s lien removal request</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>EMI Reminder</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Notifying the customer of an upcoming instalment before its due date</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Lien Removal Initiated</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>EMI Success</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Notifying the customer when the instalment is debited successfully</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Lien Removal Successful</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>The lien removal confirmation is received from the RTA</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>EMI Failed</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Lien Removal Failed</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>The lien removal request fails or is rejected by the service provider</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -1443,12 +1443,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Reminder</t>
+          <t>Sanction Letter</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+          <t>After the Sanction Letter is generated successfully (customer clicks “Sign Agreement” on the “Agreement and E-Mandate” page and the Sanction Letter is generated)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Success</t>
+          <t>Loan Agreement e-Sign</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission is successful</t>
+          <t>After the customer signs the loan agreement successfully (e-Sign at Digio – Aadhaar / VID + OTP → “Signed Successfully”)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1553,12 +1553,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Failed</t>
+          <t>LAMF Application Submit</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+          <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1578,12 +1578,12 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1608,17 +1608,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>LAMF Part Payment Confirmation</t>
+          <t>Loan Lodgement Approval</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+          <t>After the application is submitted, the OPS team approves in the backend LMS, back to back: first the Loan Account Opening approval, then the Loan Lodgement approval. This SMS is triggered when the Loan Lodgement is approved</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>LMS</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+          <t>Dear {#alp#}, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1658,57 +1658,57 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>LTV Breach Trigger (Margin Call)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Loan Account Opening / Loan Lodgement Rejection</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection, with a payment link for the charges the customer has to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1718,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>LAMF LTV Breach Liquidation</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1773,12 +1773,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>LAMF Principal Repayment Reminder</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+          <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1823,57 +1823,57 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>LAMF Liquidation for O/S</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Withdrawal Rejected</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>The withdrawal status changes to Rejected after the Operations or Treasury team rejects it</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your withdrawal request of Rs. {#alphanumeric#} for loan account {#alphanumeric#} has been rejected. For assistance, please contact our support team - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
     </row>
@@ -1883,12 +1883,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Successful Loan Tenure Completion</t>
+          <t>Loan Disbursed</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
+          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -1938,92 +1938,752 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
+          <t>EMI Reminder</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer of an upcoming instalment before its due date</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>EMI Success</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer when the instalment is debited successfully</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>EMI Failed</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>EMI Resubmission Reminder</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>EMI Resubmission Success</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer when the EMI resubmission is successful</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>EMI Resubmission Failed</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Part Payment Confirmation</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>LTV Breach Trigger (Margin Call)</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>LAMF LTV Breach Liquidation</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Principal Repayment Reminder</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Liquidation for O/S</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Successful Loan Tenure Completion</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
           <t>Loan Account Closure</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>When the loan account is closed (closed on = loan end date)</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html), discussion log DISC-176 – DISC-196.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K27"/>
+  <autoFilter ref="A1:K39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Communications: Mail table with the 21 current customer mails; Excel export with SMS and Mail sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LAMF Communications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LAMF Communications'!$A$1:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2687,4 +2689,1750 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Scenarios</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Communication Type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Sender</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Body (template)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Body (sample)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Subject</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SMS Header</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Email Verification</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>When the customer clicks Verify for the email on the KYC Verification page</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Dear Customer,
+XXXXXX is the OTP to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
+Please do not share the OTP with anyone.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Dear Customer,
+123456 is the OTP to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
+Please do not share the OTP with anyone.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mutual Fund Pledge Successful</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>After the mutual fund units are successfully pledged</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
+You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
+You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Your mutual fund pledge is successful</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Loan Sanction Letter Mail</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>After the Sanction Letter is generated. To: customer e-mail ID; CC: loandocuments@shriramcredit.in; Sanction Letter attached</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
+For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
+We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
+For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
+We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Loan Agreement Mail</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>After the loan agreement is e-signed. To: customer e-mail ID; CC: loandocuments@shriramcredit.in; signed Loan Agreement attached</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
+Your Loan ID is XXXXXXXX
+📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
+✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
+Your Loan ID is SCCLMF20261000102
+📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
+✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Initiation</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>After the loan is approved and the LAMF account is created – the customer can now initiate a withdrawal</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is XXXXXXXX.
+You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is SCCLMF20261000102.
+You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Loan Disbursal Confirmation (First Disbursement)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>When the first disbursement is credited to the customer’s bank account</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
+Loan Details:
+• Customer ID: [XXXX]
+• Loan Account ID: [XXXX]
+• Disbursement Type: &lt;&lt;Single / Multiple&gt;&gt;
+• Disbursement No.: &lt;&lt;1&gt;&gt;
+• Disbursement UTRN: [XXXX]
+• Loan Tenure: [XX months]
+• EMI Amount: ₹[XXXX]
+• First EMI Due Date: [Date]
+• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
+Repayment Schedule
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are happy to inform you that your loan amount of ₹10,000 has been credited to your bank account.
+Loan Details:
+• Customer ID: SCCL1000102
+• Loan Account ID: SCCLMF20261000102
+• Disbursement Type: Multiple
+• Disbursement No.: 1
+• Disbursement UTRN: UTIBR52026102700001
+• Loan Tenure: 12 months
+• EMI Amount: ₹88
+• First EMI Due Date: 05-11-2026
+• Balance amount available ₹1,55,26,100 (If disbursement type is MULTIPLE.)
+Repayment Schedule
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Loan Disbursal Confirmation (Subsequent Disbursement)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>When each later disbursement (disbursement type Multiple) is credited</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
+Loan Details:
+• Customer ID: [XXXX]
+• Loan Account ID: [XXXX]
+• Disbursement Type: &lt;&lt;Multiple&gt;&gt;
+• Disbursement No.: 
+• Disbursement UTRN: [XXXX]
+• Loan Tenure: [XX months]
+• EMI Amount of this disbursement for 30-day cycle: ₹[XXXX]
+• First EMI Due Date: [Date]
+• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
+Repayment Schedule (display only the residual term) – cumulative of all disbursements till date
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are happy to inform you that your loan amount of ₹20,000 has been credited to your bank account.
+Loan Details:
+• Customer ID: SCCL1000102
+• Loan Account ID: SCCLMF20261000102
+• Disbursement Type: Multiple
+• Disbursement No.: 2
+• Disbursement UTRN: UTIBR52026110200002
+• Loan Tenure: 12 months
+• EMI Amount of this disbursement for 30-day cycle: ₹175
+• First EMI Due Date: 05-12-2026
+• Balance amount available ₹1,55,06,100 (If disbursement type is MULTIPLE.)
+Repayment Schedule (display only the residual term) – cumulative of all disbursements till date
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Upcoming EMI Due Reminder</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sent 5 days before the original presentation of the EMI (routine T-5)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Here are the details of your loan:
+• Borrowed amount: ₹ 55,000
+• Outstanding amount: ₹ 55,000
+• Bank account number: XXXXXXXXXXX
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Here are the details of your loan:
+• Borrowed amount: ₹ 55,000
+• Outstanding amount: ₹ 55,000
+• Bank account number: XXXXXXXXXXX
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Reminder: Your EMI of ₹[XXXX] is due on [Date]</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>EMI Presentation Mail</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Sent one day before the EMI presentation date (routine T-1)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Here are the details of your loan:
+• Borrowed amount: ₹ 55,000
+• Outstanding amount: ₹ 55,000
+• Bank account number: XXXXXXXXXXX
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Here are the details of your loan:
+• Borrowed amount: ₹ 55,000
+• Outstanding amount: ₹ 55,000
+• Bank account number: XXXXXXXXXXX
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>EMI Presentation Alert – &lt;&lt;Date of EMI&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Successful EMI Deduction Mail</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Routine EMI clearance – the EMI is debited successfully</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are writing to confirm that your EMI of ₹[XXXX] for the loan account [Loan ID] was successfully debited on [Date] from your registered bank account.
+📄 EMI Details:
+• Loan Account Number: [Loan ID]
+• EMI Amount: ₹[XXXX]
+• Deduction Date: [Date]
+• Next EMI Due Date: [Next Date]
+Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are writing to confirm that your EMI of ₹10,000 for the loan account SCCLMF20261000102 was successfully debited on 05-11-2026 from your registered bank account.
+📄 EMI Details:
+• Loan Account Number: SCCLMF20261000102
+• EMI Amount: ₹10,000
+• Deduction Date: 05-11-2026
+• Next EMI Due Date: 05-12-2026
+Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Your EMI of ₹[XXXX] Has Been Successfully Deducted</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Instalment Failure / EMI Bounce Notification (Bounce – 1A)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>When the EMI bounces (insufficient balance); re-presented on T+5 days</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We could not process your EMI of ₹[XXXX] for the loan account [Loan ID] on [Date] due to insufficient balance.
+We will re-present the EMI on &lt;&lt;T+5 days&gt;&gt;. Please ensure your account has a sufficient balance to avoid penalties.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We could not process your EMI of ₹10,000 for the loan account SCCLMF20261000102 on 05-11-2026 due to insufficient balance.
+We will re-present the EMI on 10-11-2026. Please ensure your account has a sufficient balance to avoid penalties.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Alert: Your EMI payment failed</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Second EMI Representation Reminder (1B T-1)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Sent one day before the EMI is re-presented</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+This is to inform you that your EMI of ₹[XXXX] will be re-presented on [Date].
+Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+This is to inform you that your EMI of ₹10,000 will be re-presented on 10-11-2026.
+Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Final Reminder: EMI Re-presentation on [Date]</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Initiation of Loan Closure Procedures (2B Bounce)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>When the re-presented EMI bounces again – pledge liquidation is initiated</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Urgent: Mutual Fund Liquidation Scheduled</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Part Payment</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>When a part payment is processed successfully; the revised repayment schedule is attached</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
+Payment Summary:
+• Transaction Status: Successful
+• Amount Received: [₹XXXX Mention Amount]
+• Revised Outstanding Balance: [₹XXXX Mention Amount]
+Updated Repayment Schedule:
+As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
+Payment Summary:
+• Transaction Status: Successful
+• Amount Received: ₹5,000
+• Revised Outstanding Balance: ₹5,000
+Updated Repayment Schedule:
+As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Payment Acknowledgment: Your Shriram Credit Loan Against Mutual Funds Part Payment Has Been Processed</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Pre Closure</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>When the customer pre-closes the loan (final payment received before the end of the tenure)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation: Your Shriram Credit Loan Against Mutual Funds Has Been Closed Successfully</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Margin Call / Mutual Fund Value Drop Mail</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>When the market value of the pledged units drops and the LTV is above the limit</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+The current market value of your Mutual Fund units pledged with us has declined and current LTV is at (YY.YY)%
+We request you to make an immediate payment of ₹ (XXXX) (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of (XXXX/0.65) or For Debt MF of (XXXX/0.75)) to bring your account within the prescribed limit.
+Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
+Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
+Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your prompt attention to this matter.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+The current market value of your Mutual Fund units pledged with us has declined and current LTV is at 82.50%
+We request you to make an immediate payment of ₹ 10,000 (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of ₹15,385 or For Debt MF of ₹13,333) to bring your account within the prescribed limit.
+Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
+Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
+Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your prompt attention to this matter.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Mutual Fund Margin Shortfall</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Loan Tenure Completion (Closure Mail)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>EMI loan: when the last EMI is paid; balloon loan: when the principal outstanding is paid</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Congratulations on completing your loan journey</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>NOC / Loan Closure Certificate</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Manual trigger after the loan is closed; the NOC is attached</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan account [Loan ID] has been closed successfully.
+The No Objection Certificate (NOC) is attached for your records.
+Your Customer ID is active with us, and you may visit us for any future requirements.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+We are pleased to inform you that your loan account SCCLMF20261000102 has been closed successfully.
+The No Objection Certificate (NOC) is attached for your records.
+Your Customer ID is active with us, and you may visit us for any future requirements.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Your Loan Account [Loan ID] is closed successfully</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>LTV Breach beyond Policy Norms</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>When the LTV keeps breaching after the margin call and reaches the liquidation threshold</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
+Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
+Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Principal Repayment for Loan Closure</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>When the loan reaches maturity and the outstanding principal is unpaid – 5 working days grace period</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
+As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
+Please note that:
+• Interest at the applicable contractual rate shall continue to accrue during the grace period.
+• The outstanding amount must be repaid within the stipulated grace period.
+Please use the below link to check the details and make payment.
+{LINK}
+Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
+Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
+Thank you for your prompt attention.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
+As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
+Please note that:
+• Interest at the applicable contractual rate shall continue to accrue during the grace period.
+• The outstanding amount must be repaid within the stipulated grace period.
+Please use the below link to check the details and make payment.
+https://lamf.shriramcredit.in/user/loans/
+Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
+Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
+Thank you for your prompt attention.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Principal Repayment</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Liquidation for Outstanding Loan (after grace period)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>When the grace period for the matured loan has expired and the principal is still unpaid – liquidation is initiated. (Scenario name in the document was a pasted link – to be confirmed)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
+Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY,
+The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
+Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Communications: mails marked Available = Provided
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2833,7 +2833,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Provided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: SMS Status column (8 Not Required, rest Required); rejection without payment link; foreclosure completed SMS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$L$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="0012753B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="008A8A8A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00B42318"/>
       <sz val="11"/>
     </font>
@@ -55,7 +66,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B4C6E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -110,17 +126,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -500,6 +531,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,6 +590,11 @@
           <t>Available</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -613,6 +650,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -668,6 +710,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -723,52 +770,57 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>LAN Generated</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>When the customer clicks Continue on the Loan Application Summary page and the Loan Account Number (LAN) is generated successfully</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is {#alphanumeric#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -778,52 +830,57 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -833,52 +890,57 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Discarded</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -888,52 +950,57 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Customer-Initiated Discard</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -941,6 +1008,11 @@
       <c r="K8" s="6" t="inlineStr">
         <is>
           <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
         </is>
       </c>
     </row>
@@ -998,52 +1070,57 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Lien Marking Failed</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -1053,52 +1130,57 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Post-Pledge Journey Incomplete</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Lien marking is successful, then the customer is inactive for the configured period</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -1108,52 +1190,57 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Post-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -1163,107 +1250,117 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Application Expired – Lien Marked</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>The application reaches Day 31 without submission and the lien is still marked</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Lien Removal Request Received</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>SCCL receives and records the customer’s lien removal request</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
@@ -1273,169 +1370,189 @@
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Lien Removal Initiated</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K15" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Lien Removal Successful</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>The lien removal confirmation is received from the RTA</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="K16" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Lien Removal Failed</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>The lien removal request fails or is rejected by the service provider</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K17" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -1493,6 +1610,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1548,6 +1670,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1603,6 +1730,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1658,114 +1790,129 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Loan Account Opening / Loan Lodgement Rejection</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection, with a payment link for the charges the customer has to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Loan Account Opening / Loan Lodgement Rejection (with payment link)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITH payment link, when the customer has charges to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K22" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Loan Account Opening / Loan Lodgement Rejection (without payment link)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITHOUT payment link, when there are no charges for the customer to pay. Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -1780,157 +1927,172 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
+          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
           <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Withdrawal Rejected</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>The withdrawal status changes to Rejected after the Operations or Treasury team rejects it</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request of Rs. {#alphanumeric#} for loan account {#alphanumeric#} has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="K26" s="9" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Loan Disbursed</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="L26" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -1940,12 +2102,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>EMI Reminder</t>
+          <t>Loan Disbursed</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer of an upcoming instalment before its due date</t>
+          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1965,12 +2127,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1986,6 +2148,11 @@
       <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -1995,12 +2162,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>EMI Success</t>
+          <t>EMI Reminder</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment is debited successfully</t>
+          <t>Notifying the customer of an upcoming instalment before its due date</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2020,12 +2187,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2041,6 +2208,11 @@
       <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2050,12 +2222,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>EMI Failed</t>
+          <t>EMI Success</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+          <t>Notifying the customer when the instalment is debited successfully</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2075,12 +2247,12 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2096,6 +2268,11 @@
       <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2105,12 +2282,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Reminder</t>
+          <t>EMI Failed</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2130,12 +2307,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2151,6 +2328,11 @@
       <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2160,12 +2342,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Success</t>
+          <t>EMI Resubmission Reminder</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission is successful</t>
+          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2185,12 +2367,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2206,6 +2388,11 @@
       <c r="K31" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2215,12 +2402,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Failed</t>
+          <t>EMI Resubmission Success</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+          <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2240,12 +2427,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -2261,6 +2448,11 @@
       <c r="K32" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2270,12 +2462,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>LAMF Part Payment Confirmation</t>
+          <t>EMI Resubmission Failed</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2295,12 +2487,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2316,6 +2508,11 @@
       <c r="K33" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2325,12 +2522,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>LTV Breach Trigger (Margin Call)</t>
+          <t>LAMF Part Payment Confirmation</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
+          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2350,12 +2547,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2371,6 +2568,11 @@
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2380,12 +2582,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>LAMF LTV Breach Liquidation</t>
+          <t>LTV Breach Trigger (Margin Call)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2405,12 +2607,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2426,6 +2628,11 @@
       <c r="K35" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2435,12 +2642,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>LAMF Principal Repayment Reminder</t>
+          <t>LAMF LTV Breach Liquidation</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2460,12 +2667,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2481,6 +2688,11 @@
       <c r="K36" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2490,12 +2702,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>LAMF Liquidation for O/S</t>
+          <t>LAMF Principal Repayment Reminder</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2515,12 +2727,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2536,6 +2748,11 @@
       <c r="K37" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2545,147 +2762,284 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
+          <t>LAMF Liquidation for O/S</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Foreclosure Completed</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
           <t>Successful Loan Tenure Completion</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Loan Account Closure</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>When the loan account is closed (closed on = loan end date)</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>Rows in grey (Status = "Not Required") are kept for reference only; they will not be sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K39"/>
+  <autoFilter ref="A1:L41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2697,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4396,35 +4750,42 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Rows in grey (Status = "Not Required") are kept for reference only; they will not be sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>

</xml_diff>

<commit_message>
Communications SMS table: Mail Communication Available, Mail Subject Line, Mail Content columns (18 SMS mapped to their mail)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$O$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -532,6 +532,9 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="80" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -595,6 +598,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Communication Available</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Subject Line</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Content</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -645,14 +663,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -705,14 +738,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -765,14 +813,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -825,14 +888,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -885,14 +963,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -945,14 +1038,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1005,14 +1113,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1065,14 +1188,35 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Your mutual fund pledge is successful</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
+You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -1125,14 +1269,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1185,14 +1344,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1245,14 +1419,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1305,14 +1494,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L13" s="11" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1365,14 +1569,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>Not Required</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1425,14 +1644,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L15" s="11" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1485,14 +1719,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L16" s="11" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1545,14 +1794,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L17" s="11" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1605,14 +1869,38 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
+For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
+We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -1665,14 +1953,39 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
+Your Loan ID is XXXXXXXX
+📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
+✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -1725,14 +2038,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1785,14 +2113,37 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is XXXXXXXX.
+You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -1845,14 +2196,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L22" s="11" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1905,14 +2271,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L23" s="11" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1965,14 +2346,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2025,14 +2421,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2085,14 +2496,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K26" s="9" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L26" s="11" t="inlineStr">
+      <c r="L26" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2145,14 +2571,51 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
+Loan Details:
+• Customer ID: [XXXX]
+• Loan Account ID: [XXXX]
+• Disbursement Type: &lt;&lt;Single / Multiple&gt;&gt;
+• Disbursement No.: &lt;&lt;1&gt;&gt;
+• Disbursement UTRN: [XXXX]
+• Loan Tenure: [XX months]
+• EMI Amount: ₹[XXXX]
+• First EMI Due Date: [Date]
+• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
+Repayment Schedule
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2205,14 +2668,40 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Reminder: Your EMI of ₹[XXXX] is due on [Date]</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Here are the details of your loan:
+• Borrowed amount: ₹ 55,000
+• Outstanding amount: ₹ 55,000
+• Bank account number: XXXXXXXXXXX
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2265,14 +2754,41 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Your EMI of ₹[XXXX] Has Been Successfully Deducted</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are writing to confirm that your EMI of ₹[XXXX] for the loan account [Loan ID] was successfully debited on [Date] from your registered bank account.
+📄 EMI Details:
+• Loan Account Number: [Loan ID]
+• EMI Amount: ₹[XXXX]
+• Deduction Date: [Date]
+• Next EMI Due Date: [Next Date]
+Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2325,14 +2841,37 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>Alert: Your EMI payment failed</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We could not process your EMI of ₹[XXXX] for the loan account [Loan ID] on [Date] due to insufficient balance.
+We will re-present the EMI on &lt;&lt;T+5 days&gt;&gt;. Please ensure your account has a sufficient balance to avoid penalties.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2385,14 +2924,36 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Final Reminder: EMI Re-presentation on [Date]</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+This is to inform you that your EMI of ₹[XXXX] will be re-presented on [Date].
+Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2445,14 +3006,29 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2505,14 +3081,35 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Urgent: Mutual Fund Liquidation Scheduled</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2565,14 +3162,42 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L34" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Payment Acknowledgment: Your Shriram Credit Loan Against Mutual Funds Part Payment Has Been Processed</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
+Payment Summary:
+• Transaction Status: Successful
+• Amount Received: [₹XXXX Mention Amount]
+• Revised Outstanding Balance: [₹XXXX Mention Amount]
+Updated Repayment Schedule:
+As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2625,14 +3250,39 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Mutual Fund Margin Shortfall</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+The current market value of your Mutual Fund units pledged with us has declined and current LTV is at (YY.YY)%
+We request you to make an immediate payment of ₹ (XXXX) (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of (XXXX/0.65) or For Debt MF of (XXXX/0.75)) to bring your account within the prescribed limit.
+Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
+Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
+Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your prompt attention to this matter.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2685,14 +3335,38 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L36" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
+Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2745,14 +3419,43 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L37" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Principal Repayment</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
+As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
+Please note that:
+• Interest at the applicable contractual rate shall continue to accrue during the grace period.
+• The outstanding amount must be repaid within the stipulated grace period.
+Please use the below link to check the details and make payment.
+{LINK}
+Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
+Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
+Thank you for your prompt attention.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2805,14 +3508,38 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L38" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
+Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2865,14 +3592,46 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K39" s="9" t="inlineStr">
+      <c r="K39" s="11" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L39" s="11" t="inlineStr">
+      <c r="L39" s="9" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation: Your Shriram Credit Loan Against Mutual Funds Has Been Closed Successfully</t>
+        </is>
+      </c>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2925,14 +3684,46 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr">
+      <c r="K40" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L40" s="4" t="inlineStr">
+      <c r="L40" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>Congratulations on completing your loan journey</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
+We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process:
+As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
+• Timeline: The lien will be removed within 2 to 3 working days.
+• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
+Next Steps:
+No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
+Important Information:
+• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
+• In case the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -2985,14 +3776,37 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K41" s="3" t="inlineStr">
+      <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr">
+      <c r="L41" s="3" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Your Loan Account [Loan ID] is closed successfully</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>Dear [Customer Name],
+We are pleased to inform you that your loan account [Loan ID] has been closed successfully.
+The No Objection Certificate (NOC) is attached for your records.
+Your Customer ID is active with us, and you may visit us for any future requirements.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3853,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:O41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Communications SMS table: mail column values cleared (to be filled from the owner's list)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -673,21 +673,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -748,21 +736,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -823,21 +799,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M4" s="3" t="inlineStr"/>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -898,21 +862,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M5" s="6" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
+      <c r="O5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -973,21 +925,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M6" s="6" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr"/>
+      <c r="O6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -1048,21 +988,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -1123,21 +1051,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M8" s="6" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr"/>
+      <c r="O8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1198,27 +1114,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>Your mutual fund pledge is successful</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
-You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -1279,21 +1177,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M10" s="6" t="inlineStr"/>
+      <c r="N10" s="6" t="inlineStr"/>
+      <c r="O10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -1354,21 +1240,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M11" s="6" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1429,21 +1303,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M12" s="6" t="inlineStr"/>
+      <c r="N12" s="6" t="inlineStr"/>
+      <c r="O12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -1504,21 +1366,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N13" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O13" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M13" s="9" t="inlineStr"/>
+      <c r="N13" s="9" t="inlineStr"/>
+      <c r="O13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1579,21 +1429,9 @@
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N14" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M14" s="6" t="inlineStr"/>
+      <c r="N14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -1654,21 +1492,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N15" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O15" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M15" s="9" t="inlineStr"/>
+      <c r="N15" s="9" t="inlineStr"/>
+      <c r="O15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1729,21 +1555,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M16" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N16" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O16" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M16" s="9" t="inlineStr"/>
+      <c r="N16" s="9" t="inlineStr"/>
+      <c r="O16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1804,21 +1618,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N17" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M17" s="9" t="inlineStr"/>
+      <c r="N17" s="9" t="inlineStr"/>
+      <c r="O17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1879,30 +1681,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N18" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
-For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
-We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1963,31 +1744,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
-Your Loan ID is XXXXXXXX
-📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
-✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2048,21 +1807,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2123,29 +1870,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N21" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal Initiation: Successful LAMF Account Creation – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is XXXXXXXX.
-You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -2206,21 +1933,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M22" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N22" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O22" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M22" s="9" t="inlineStr"/>
+      <c r="N22" s="9" t="inlineStr"/>
+      <c r="O22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -2281,21 +1996,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M23" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N23" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O23" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M23" s="9" t="inlineStr"/>
+      <c r="N23" s="9" t="inlineStr"/>
+      <c r="O23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2356,21 +2059,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr"/>
+      <c r="O24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2431,21 +2122,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M25" s="3" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
@@ -2506,21 +2185,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M26" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N26" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O26" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M26" s="9" t="inlineStr"/>
+      <c r="N26" s="9" t="inlineStr"/>
+      <c r="O26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2581,43 +2248,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="inlineStr">
-        <is>
-          <t>Loan disbursed to your account</t>
-        </is>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
-Loan Details:
-• Customer ID: [XXXX]
-• Loan Account ID: [XXXX]
-• Disbursement Type: &lt;&lt;Single / Multiple&gt;&gt;
-• Disbursement No.: &lt;&lt;1&gt;&gt;
-• Disbursement UTRN: [XXXX]
-• Loan Tenure: [XX months]
-• EMI Amount: ₹[XXXX]
-• First EMI Due Date: [Date]
-• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
-Repayment Schedule
-Repayment Date | Repayment Amount
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M27" s="3" t="inlineStr"/>
+      <c r="N27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2678,32 +2311,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="inlineStr">
-        <is>
-          <t>Reminder: Your EMI of ₹[XXXX] is due on [Date]</t>
-        </is>
-      </c>
-      <c r="O28" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
-Here are the details of your loan:
-• Borrowed amount: ₹ 55,000
-• Outstanding amount: ₹ 55,000
-• Bank account number: XXXXXXXXXXX
-Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
-Thank you for your cooperation.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M28" s="3" t="inlineStr"/>
+      <c r="N28" s="3" t="inlineStr"/>
+      <c r="O28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2764,33 +2374,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N29" s="3" t="inlineStr">
-        <is>
-          <t>Your EMI of ₹[XXXX] Has Been Successfully Deducted</t>
-        </is>
-      </c>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are writing to confirm that your EMI of ₹[XXXX] for the loan account [Loan ID] was successfully debited on [Date] from your registered bank account.
-📄 EMI Details:
-• Loan Account Number: [Loan ID]
-• EMI Amount: ₹[XXXX]
-• Deduction Date: [Date]
-• Next EMI Due Date: [Next Date]
-Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M29" s="3" t="inlineStr"/>
+      <c r="N29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2851,29 +2437,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr">
-        <is>
-          <t>Alert: Your EMI payment failed</t>
-        </is>
-      </c>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We could not process your EMI of ₹[XXXX] for the loan account [Loan ID] on [Date] due to insufficient balance.
-We will re-present the EMI on &lt;&lt;T+5 days&gt;&gt;. Please ensure your account has a sufficient balance to avoid penalties.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M30" s="3" t="inlineStr"/>
+      <c r="N30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2934,28 +2500,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N31" s="3" t="inlineStr">
-        <is>
-          <t>Final Reminder: EMI Re-presentation on [Date]</t>
-        </is>
-      </c>
-      <c r="O31" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-This is to inform you that your EMI of ₹[XXXX] will be re-presented on [Date].
-Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M31" s="3" t="inlineStr"/>
+      <c r="N31" s="3" t="inlineStr"/>
+      <c r="O31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3016,21 +2563,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O32" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M32" s="3" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr"/>
+      <c r="O32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3091,27 +2626,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>Urgent: Mutual Fund Liquidation Scheduled</t>
-        </is>
-      </c>
-      <c r="O33" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr"/>
+      <c r="O33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3172,34 +2689,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N34" s="3" t="inlineStr">
-        <is>
-          <t>Payment Acknowledgment: Your Shriram Credit Loan Against Mutual Funds Part Payment Has Been Processed</t>
-        </is>
-      </c>
-      <c r="O34" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
-Payment Summary:
-• Transaction Status: Successful
-• Amount Received: [₹XXXX Mention Amount]
-• Revised Outstanding Balance: [₹XXXX Mention Amount]
-Updated Repayment Schedule:
-As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M34" s="3" t="inlineStr"/>
+      <c r="N34" s="3" t="inlineStr"/>
+      <c r="O34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3260,31 +2752,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Mutual Fund Margin Shortfall</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-The current market value of your Mutual Fund units pledged with us has declined and current LTV is at (YY.YY)%
-We request you to make an immediate payment of ₹ (XXXX) (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of (XXXX/0.65) or For Debt MF of (XXXX/0.75)) to bring your account within the prescribed limit.
-Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
-Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
-Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your prompt attention to this matter.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="inlineStr"/>
+      <c r="O35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3345,30 +2815,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach</t>
-        </is>
-      </c>
-      <c r="O36" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
-Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="inlineStr"/>
+      <c r="O36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3429,35 +2878,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N37" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Principal Repayment</t>
-        </is>
-      </c>
-      <c r="O37" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
-As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
-Please note that:
-• Interest at the applicable contractual rate shall continue to accrue during the grace period.
-• The outstanding amount must be repaid within the stipulated grace period.
-Please use the below link to check the details and make payment.
-{LINK}
-Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
-Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
-Thank you for your prompt attention.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" s="3" t="inlineStr"/>
+      <c r="O37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3518,30 +2941,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N38" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan</t>
-        </is>
-      </c>
-      <c r="O38" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
-Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" s="3" t="inlineStr"/>
+      <c r="O38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
@@ -3602,38 +3004,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M39" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N39" s="9" t="inlineStr">
-        <is>
-          <t>Loan Pre-Closure Confirmation: Your Shriram Credit Loan Against Mutual Funds Has Been Closed Successfully</t>
-        </is>
-      </c>
-      <c r="O39" s="9" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M39" s="9" t="inlineStr"/>
+      <c r="N39" s="9" t="inlineStr"/>
+      <c r="O39" s="9" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3694,38 +3067,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N40" s="3" t="inlineStr">
-        <is>
-          <t>Congratulations on completing your loan journey</t>
-        </is>
-      </c>
-      <c r="O40" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M40" s="3" t="inlineStr"/>
+      <c r="N40" s="3" t="inlineStr"/>
+      <c r="O40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3786,29 +3130,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N41" s="3" t="inlineStr">
-        <is>
-          <t>Your Loan Account [Loan ID] is closed successfully</t>
-        </is>
-      </c>
-      <c r="O41" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan account [Loan ID] has been closed successfully.
-The No Objection Certificate (NOC) is attached for your records.
-Your Customer ID is active with us, and you may visit us for any future requirements.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
+      <c r="M41" s="3" t="inlineStr"/>
+      <c r="N41" s="3" t="inlineStr"/>
+      <c r="O41" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Communications: Email Verification mail row; SMS table columns renamed and re-ordered with mail subject / content / available / status columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$Q$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="008A8A8A"/>
       <sz val="11"/>
     </font>
@@ -54,6 +60,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00B42318"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008A8A8A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -115,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -129,13 +141,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -144,14 +162,17 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -517,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -529,12 +550,14 @@
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="80" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -570,47 +593,57 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Content Structure</t>
+          <t>SMS Content Structure</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Actual Content</t>
+          <t>Actual SMS Content</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>SMS Header</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SMS Available</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SMS Status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Subject Structure</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Mail Subject</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SMS Header</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Mail Communication Available</t>
-        </is>
-      </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Mail Subject Line</t>
+          <t>Mail Content Structure</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Mail Content</t>
+          <t>Actual Mail Content</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Available</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Status</t>
         </is>
       </c>
     </row>
@@ -655,27 +688,25 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L2" s="3" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -718,27 +749,25 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -781,909 +810,921 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>LAN Generated</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>When the customer clicks Continue on the Loan Application Summary page and the Loan Account Number (LAN) is generated successfully</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is {#alphanumeric#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Email Verification</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>On the KYC Verification page (LOS step 9, after the Application Summary): the customer enters the email address and clicks Verify, and the OTP is sent to that email</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>123456 – Your Email Verification OTP for Shriram Credit LAMF</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>E-Mail Verification
+Dear {{CUSTOMER_NAME}},
+One-Time Password
+{{OTP}}
+Please do not share the OTP with anyone.
+Use the OTP above to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>E-Mail Verification
+Dear AZHAGARSAMY,
+One-Time Password
+123456
+Please do not share the OTP with anyone.
+Use the OTP above to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Provided</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Pre-Pledge Application Expiry Reminder</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr"/>
-      <c r="O5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Pre-Pledge Application Expiry Reminder</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr"/>
+      <c r="P7" s="7" t="inlineStr"/>
+      <c r="Q7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Pre-Pledge Application Discarded</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="6" t="inlineStr"/>
-      <c r="O6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Pre-Pledge Application Discarded</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr"/>
+      <c r="N8" s="7" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr"/>
+      <c r="P8" s="7" t="inlineStr"/>
+      <c r="Q8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Customer-Initiated Discard</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Customer-Initiated Discard</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr"/>
+      <c r="P9" s="7" t="inlineStr"/>
+      <c r="Q9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Pledging of Mutual Fund</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>After the mutual fund units are successfully pledged on the “Pledging of Mutual Fund” page (Pledge Securities → MF Central OTP → “Successfully pledged!”)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Lien Marking Failed</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr"/>
-      <c r="N8" s="6" t="inlineStr"/>
-      <c r="O8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Pledging of Mutual Fund</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>After the mutual fund units are successfully pledged on the “Pledging of Mutual Fund” page (Pledge Securities → MF Central OTP → “Successfully pledged!”)</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr"/>
+      <c r="P11" s="7" t="inlineStr"/>
+      <c r="Q11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Post-Pledge Journey Incomplete</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Lien marking is successful, then the customer is inactive for the configured period</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr"/>
+      <c r="N12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr"/>
+      <c r="P12" s="7" t="inlineStr"/>
+      <c r="Q12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Post-Pledge Application Expiry Reminder</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr"/>
+      <c r="P13" s="7" t="inlineStr"/>
+      <c r="Q13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Application Expired – Lien Marked</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>The application reaches Day 31 without submission and the lien is still marked</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr"/>
-      <c r="N9" s="3" t="inlineStr"/>
-      <c r="O9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Lien Marking Failed</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr"/>
+      <c r="M14" s="11" t="inlineStr"/>
+      <c r="N14" s="11" t="inlineStr"/>
+      <c r="O14" s="11" t="inlineStr"/>
+      <c r="P14" s="11" t="inlineStr"/>
+      <c r="Q14" s="14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Lien Removal Request Received</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>SCCL receives and records the customer’s lien removal request</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>Not Required</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr"/>
-      <c r="N10" s="6" t="inlineStr"/>
-      <c r="O10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Post-Pledge Journey Incomplete</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Lien marking is successful, then the customer is inactive for the configured period</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr"/>
+      <c r="P15" s="7" t="inlineStr"/>
+      <c r="Q15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Lien Removal Initiated</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr"/>
-      <c r="O11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Post-Pledge Application Expiry Reminder</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr"/>
+      <c r="M16" s="11" t="inlineStr"/>
+      <c r="N16" s="11" t="inlineStr"/>
+      <c r="O16" s="11" t="inlineStr"/>
+      <c r="P16" s="11" t="inlineStr"/>
+      <c r="Q16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Lien Removal Successful</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>The lien removal confirmation is received from the RTA</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="6" t="inlineStr"/>
-      <c r="O12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Application Expired – Lien Marked</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>The application reaches Day 31 without submission and the lien is still marked</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr"/>
+      <c r="M17" s="11" t="inlineStr"/>
+      <c r="N17" s="11" t="inlineStr"/>
+      <c r="O17" s="11" t="inlineStr"/>
+      <c r="P17" s="11" t="inlineStr"/>
+      <c r="Q17" s="14" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Lien Removal Failed</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>The lien removal request fails or is rejected by the service provider</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K13" s="11" t="inlineStr">
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L13" s="9" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="9" t="inlineStr"/>
-      <c r="O13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Lien Removal Request Received</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>SCCL receives and records the customer’s lien removal request</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>No – to be created</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="6" t="inlineStr"/>
-      <c r="O14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Lien Removal Initiated</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>No – to be created</t>
-        </is>
-      </c>
-      <c r="L15" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M15" s="9" t="inlineStr"/>
-      <c r="N15" s="9" t="inlineStr"/>
-      <c r="O15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Lien Removal Successful</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>The lien removal confirmation is received from the RTA</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>No – to be created</t>
-        </is>
-      </c>
-      <c r="L16" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M16" s="9" t="inlineStr"/>
-      <c r="N16" s="9" t="inlineStr"/>
-      <c r="O16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Lien Removal Failed</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>The lien removal request fails or is rejected by the service provider</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>No – to be created</t>
-        </is>
-      </c>
-      <c r="L17" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M17" s="9" t="inlineStr"/>
-      <c r="N17" s="9" t="inlineStr"/>
-      <c r="O17" s="9" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Sanction Letter</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>After the Sanction Letter is generated successfully (customer clicks “Sign Agreement” on the “Agreement and E-Mandate” page and the Sanction Letter is generated)</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L18" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-      <c r="O18" s="3" t="inlineStr"/>
+      <c r="L18" s="11" t="inlineStr"/>
+      <c r="M18" s="11" t="inlineStr"/>
+      <c r="N18" s="11" t="inlineStr"/>
+      <c r="O18" s="11" t="inlineStr"/>
+      <c r="P18" s="11" t="inlineStr"/>
+      <c r="Q18" s="14" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1691,12 +1732,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Loan Agreement e-Sign</t>
+          <t>Sanction Letter</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>After the customer signs the loan agreement successfully (e-Sign at Digio – Aadhaar / VID + OTP → “Signed Successfully”)</t>
+          <t>After the Sanction Letter is generated successfully (customer clicks “Sign Agreement” on the “Agreement and E-Mandate” page and the Sanction Letter is generated)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1716,37 +1757,35 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1754,12 +1793,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>LAMF Application Submit</t>
+          <t>Loan Agreement e-Sign</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
+          <t>After the customer signs the loan agreement successfully (e-Sign at Digio – Aadhaar / VID + OTP → “Signed Successfully”)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1779,37 +1818,35 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L20" s="3" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr"/>
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr"/>
+      <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1817,17 +1854,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Loan Lodgement Approval</t>
+          <t>LAMF Application Submit</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>After the application is submitted, the OPS team approves in the backend LMS, back to back: first the Loan Account Opening approval, then the Loan Lodgement approval. This SMS is triggered when the Loan Lodgement is approved</t>
+          <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>LMS</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1842,226 +1879,218 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- https://lamf.shriramcredit.in/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L21" s="3" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr"/>
       <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Loan Lodgement Approval</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>After the application is submitted, the OPS team approves in the backend LMS, back to back: first the Loan Account Opening approval, then the Loan Lodgement approval. This SMS is triggered when the Loan Lodgement is approved</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- {#urg#} - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- https://lamf.shriramcredit.in/ - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr"/>
+      <c r="O22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (with payment link)</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITH payment link, when the customer has charges to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K22" s="11" t="inlineStr">
+      <c r="J23" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L22" s="9" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M22" s="9" t="inlineStr"/>
-      <c r="N22" s="9" t="inlineStr"/>
-      <c r="O22" s="9" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="L23" s="11" t="inlineStr"/>
+      <c r="M23" s="11" t="inlineStr"/>
+      <c r="N23" s="11" t="inlineStr"/>
+      <c r="O23" s="11" t="inlineStr"/>
+      <c r="P23" s="11" t="inlineStr"/>
+      <c r="Q23" s="14" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (without payment link)</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITHOUT payment link, when there are no charges for the customer to pay. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
+      <c r="J24" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L23" s="9" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M23" s="9" t="inlineStr"/>
-      <c r="N23" s="9" t="inlineStr"/>
-      <c r="O23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr"/>
-      <c r="N24" s="3" t="inlineStr"/>
-      <c r="O24" s="3" t="inlineStr"/>
+      <c r="L24" s="11" t="inlineStr"/>
+      <c r="M24" s="11" t="inlineStr"/>
+      <c r="N24" s="11" t="inlineStr"/>
+      <c r="O24" s="11" t="inlineStr"/>
+      <c r="P24" s="11" t="inlineStr"/>
+      <c r="Q24" s="14" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2074,7 +2103,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
+          <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -2094,163 +2123,157 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
+          <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
+          <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L25" s="3" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr"/>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr"/>
+      <c r="N26" s="3" t="inlineStr"/>
+      <c r="O26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Withdrawal Rejected</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>The withdrawal status changes to Rejected after the Operations or Treasury team rejects it</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request of Rs. {#alphanumeric#} for loan account {#alphanumeric#} has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="10" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L26" s="9" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M26" s="9" t="inlineStr"/>
-      <c r="N26" s="9" t="inlineStr"/>
-      <c r="O26" s="9" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Loan Disbursed</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr"/>
-      <c r="N27" s="3" t="inlineStr"/>
-      <c r="O27" s="3" t="inlineStr"/>
+      <c r="L27" s="11" t="inlineStr"/>
+      <c r="M27" s="11" t="inlineStr"/>
+      <c r="N27" s="11" t="inlineStr"/>
+      <c r="O27" s="11" t="inlineStr"/>
+      <c r="P27" s="11" t="inlineStr"/>
+      <c r="Q27" s="14" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2258,12 +2281,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>EMI Reminder</t>
+          <t>Loan Disbursed</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer of an upcoming instalment before its due date</t>
+          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2283,37 +2306,35 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L28" s="3" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr"/>
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2321,12 +2342,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>EMI Success</t>
+          <t>EMI Reminder</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment is debited successfully</t>
+          <t>Notifying the customer of an upcoming instalment before its due date</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2346,37 +2367,35 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L29" s="3" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr"/>
       <c r="N29" s="3" t="inlineStr"/>
       <c r="O29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2384,12 +2403,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>EMI Failed</t>
+          <t>EMI Success</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+          <t>Notifying the customer when the instalment is debited successfully</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2409,37 +2428,35 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L30" s="3" t="inlineStr"/>
       <c r="M30" s="3" t="inlineStr"/>
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2447,12 +2464,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Reminder</t>
+          <t>EMI Failed</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2472,37 +2489,35 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L31" s="3" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr"/>
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="inlineStr"/>
+      <c r="Q31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2510,12 +2525,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Success</t>
+          <t>EMI Resubmission Reminder</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission is successful</t>
+          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2535,37 +2550,35 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L32" s="3" t="inlineStr"/>
       <c r="M32" s="3" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr"/>
       <c r="O32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2573,12 +2586,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Failed</t>
+          <t>EMI Resubmission Success</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+          <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2598,37 +2611,35 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr"/>
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr"/>
+      <c r="P33" s="3" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2636,12 +2647,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>LAMF Part Payment Confirmation</t>
+          <t>EMI Resubmission Failed</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2661,37 +2672,35 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L34" s="3" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr"/>
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2699,12 +2708,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>LTV Breach Trigger (Margin Call)</t>
+          <t>LAMF Part Payment Confirmation</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
+          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2724,37 +2733,35 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L35" s="3" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr"/>
+      <c r="P35" s="3" t="inlineStr"/>
+      <c r="Q35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2762,12 +2769,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>LAMF LTV Breach Liquidation</t>
+          <t>LTV Breach Trigger (Margin Call)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2787,37 +2794,35 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="J36" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L36" s="3" t="inlineStr"/>
       <c r="M36" s="3" t="inlineStr"/>
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr"/>
+      <c r="P36" s="3" t="inlineStr"/>
+      <c r="Q36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2825,12 +2830,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>LAMF Principal Repayment Reminder</t>
+          <t>LAMF LTV Breach Liquidation</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2850,37 +2855,35 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L37" s="3" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L37" s="3" t="inlineStr"/>
       <c r="M37" s="3" t="inlineStr"/>
       <c r="N37" s="3" t="inlineStr"/>
       <c r="O37" s="3" t="inlineStr"/>
+      <c r="P37" s="3" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2888,12 +2891,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>LAMF Liquidation for O/S</t>
+          <t>LAMF Principal Repayment Reminder</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2913,163 +2916,157 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L38" s="3" t="inlineStr"/>
       <c r="M38" s="3" t="inlineStr"/>
       <c r="N38" s="3" t="inlineStr"/>
       <c r="O38" s="3" t="inlineStr"/>
+      <c r="P38" s="3" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="n">
+      <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Liquidation for O/S</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="3" t="inlineStr"/>
+      <c r="O39" s="3" t="inlineStr"/>
+      <c r="P39" s="3" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Foreclosure Completed</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="H39" s="9" t="inlineStr">
+      <c r="H40" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I39" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J39" s="10" t="inlineStr">
+      <c r="I40" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K39" s="11" t="inlineStr">
+      <c r="J40" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="L39" s="9" t="inlineStr">
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="M39" s="9" t="inlineStr"/>
-      <c r="N39" s="9" t="inlineStr"/>
-      <c r="O39" s="9" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Successful Loan Tenure Completion</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L40" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="3" t="inlineStr"/>
-      <c r="O40" s="3" t="inlineStr"/>
+      <c r="L40" s="11" t="inlineStr"/>
+      <c r="M40" s="11" t="inlineStr"/>
+      <c r="N40" s="11" t="inlineStr"/>
+      <c r="O40" s="11" t="inlineStr"/>
+      <c r="P40" s="11" t="inlineStr"/>
+      <c r="Q40" s="14" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3077,12 +3074,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Loan Account Closure</t>
+          <t>Successful Loan Tenure Completion</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>When the loan account is closed (closed on = loan end date)</t>
+          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -3102,82 +3099,141 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L41" s="3" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
+      <c r="L41" s="3" t="inlineStr"/>
       <c r="M41" s="3" t="inlineStr"/>
       <c r="N41" s="3" t="inlineStr"/>
       <c r="O41" s="3" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="P41" s="3" t="inlineStr"/>
+      <c r="Q41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Loan Account Closure</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>When the loan account is closed (closed on = loan end date)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr"/>
+      <c r="N42" s="3" t="inlineStr"/>
+      <c r="O42" s="3" t="inlineStr"/>
+      <c r="P42" s="3" t="inlineStr"/>
+      <c r="Q42" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>Rows in grey (Status = "Not Required") are kept for reference only; they will not be sent.</t>
-        </is>
-      </c>
-    </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O41"/>
+  <autoFilter ref="A1:Q42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4888,42 +4944,42 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Rows in grey (Status = "Not Required") are kept for reference only; they will not be sent.</t>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>

</xml_diff>

<commit_message>
Communications: Sender before Communication Type
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -583,12 +583,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Sender</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Communication Type</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sender</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -729,12 +729,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -790,12 +790,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1076,12 +1076,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1137,12 +1137,12 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1198,12 +1198,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1564,12 +1564,12 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1686,12 +1686,12 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1869,12 +1869,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1991,12 +1991,12 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -2113,12 +2113,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2235,12 +2235,12 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -2296,12 +2296,12 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -2357,12 +2357,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2540,12 +2540,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -2601,12 +2601,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2662,12 +2662,12 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -2723,12 +2723,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2784,12 +2784,12 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -2845,12 +2845,12 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2906,12 +2906,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2967,12 +2967,12 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -3028,12 +3028,12 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -3089,12 +3089,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
           <t>SMS</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -3284,12 +3284,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Sender</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Communication Type</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sender</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3339,12 +3339,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -3406,12 +3406,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3473,12 +3473,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3546,12 +3546,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3621,12 +3621,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3692,12 +3692,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -3791,12 +3791,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3890,12 +3890,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3967,12 +3967,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -4044,12 +4044,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -4123,12 +4123,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -4194,12 +4194,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -4263,12 +4263,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -4330,12 +4330,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -4411,12 +4411,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -4500,12 +4500,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4575,12 +4575,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -4664,12 +4664,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4735,12 +4735,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -4808,12 +4808,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -4891,12 +4891,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
           <t>Mail</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Communications: Email Verification Mail Available = Yes with View link to the HTML mail template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -985,7 +985,8 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Yes
+View mail</t>
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
@@ -3234,6 +3235,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Q42"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Communications: pledge, sanction letter and loan agreement rows now SMS + Mail with the owner's HTML templates (View links)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1204,7 +1204,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1232,12 +1232,53 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
-      <c r="N10" s="3" t="inlineStr"/>
-      <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="3" t="inlineStr"/>
-      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Your mutual fund pledge is successful</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Your mutual fund pledge is successful</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Mutual Fund Pledge Successful
+Dear {{CUSTOMER_NAME}},
+✓ Pledge Successfully Completed
+Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
+You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Mutual Fund Pledge Successful
+Dear AZHAGARSAMY,
+✓ Pledge Successfully Completed
+Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
+You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -1753,7 +1794,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1781,12 +1822,63 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr"/>
-      <c r="O19" s="3" t="inlineStr"/>
-      <c r="P19" s="3" t="inlineStr"/>
-      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Sanction Letter – AZHAGARSAMY SUBBURAJ</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>To: Customer Email ID
+CC: loandocuments@shriramcredit.in
+Attachment: Loan Sanction Letter PDF
+Loan Sanction Letter
+Dear {{CUSTOMER_NAME}},
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
+📄 Loan Sanction Letter attached — please find the complete details of your approved loan including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
+We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>To: Customer Email ID
+CC: loandocuments@shriramcredit.in
+Attachment: Loan Sanction Letter PDF
+Loan Sanction Letter
+Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
+📄 Loan Sanction Letter attached — please find the complete details of your approved loan including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
+We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1814,7 +1906,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1842,12 +1934,67 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
-      <c r="N20" s="3" t="inlineStr"/>
-      <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="3" t="inlineStr"/>
-      <c r="Q20" s="5" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>SCCL Loan Agreement – AZHAGARSAMY SUBBURAJ</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>To: Customer Email ID
+CC: loandocuments@shriramcredit.in
+Attachment: Digitally signed Loan Agreement PDF
+Loan Agreement
+Dear {{CUSTOMER_NAME}},
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
+Your Loan ID
+{{LOAN_ID}}
+📄 Digitally signed loan agreement is attached. Please review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
+✓ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>To: Customer Email ID
+CC: loandocuments@shriramcredit.in
+Attachment: Digitally signed Loan Agreement PDF
+Loan Agreement
+Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
+Your Loan ID
+SCCLMF20261000102
+📄 Digitally signed loan agreement is attached. Please review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
+✓ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -3237,6 +3384,9 @@
   <autoFilter ref="A1:Q42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: withdrawal OTP row now SMS + Mail with the owner's HTML template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2266,7 +2266,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2294,12 +2294,55 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr"/>
-      <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="3" t="inlineStr"/>
-      <c r="Q25" s="5" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>{{OTP}} – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>123456 – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Verification
+Dear {{CUSTOMER_NAME}},
+One-Time Password
+{{OTP}}
+Please do not share the OTP with anyone.
+Use the OTP above to confirm the withdrawal of ₹{{WITHDRAWAL_AMOUNT}} from your Loan Against Mutual Fund.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Verification
+Dear AZHAGARSAMY,
+One-Time Password
+123456
+Please do not share the OTP with anyone.
+Use the OTP above to confirm the withdrawal of ₹10,000 from your Loan Against Mutual Fund.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -3387,6 +3430,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: loan lodgement approval row now SMS + Mail (withdrawal initiation template)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2083,7 +2083,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -2111,12 +2111,59 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
-      <c r="N22" s="3" t="inlineStr"/>
-      <c r="O22" s="3" t="inlineStr"/>
-      <c r="P22" s="3" t="inlineStr"/>
-      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – {{CUSTOMER_FULL_NAME}}</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – AZHAGARSAMY SUBBURAJ</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Loan Approved
+Dear {{CUSTOMER_NAME}},
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is {{LOAN_ID}}.
+You can now proceed to initiate the withdrawal request for the approved amount at:
+[Initiate Withdrawal Request]
+or visit: {{Link}}
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>Loan Approved
+Dear AZHAGARSAMY,
+We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is SCCLMF20261000102.
+You can now proceed to initiate the withdrawal request for the approved amount at:
+[Initiate Withdrawal Request]
+or visit: https://lamf.shriramcredit.in/
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -3430,7 +3477,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Remarks column (pledge mail timing remark)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -538,15 +538,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -558,6 +558,7 @@
     <col width="70" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,6 +645,11 @@
       <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Mail Status</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
         </is>
       </c>
     </row>
@@ -707,6 +713,7 @@
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="3" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -768,6 +775,7 @@
       <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -829,6 +837,7 @@
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -890,6 +899,7 @@
       <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="7" t="inlineStr"/>
       <c r="Q5" s="9" t="inlineStr"/>
+      <c r="R5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -994,6 +1004,7 @@
           <t>Required</t>
         </is>
       </c>
+      <c r="R6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -1055,6 +1066,7 @@
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr"/>
       <c r="Q7" s="9" t="inlineStr"/>
+      <c r="R7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -1116,6 +1128,7 @@
       <c r="O8" s="7" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr"/>
       <c r="Q8" s="9" t="inlineStr"/>
+      <c r="R8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1177,6 +1190,7 @@
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr"/>
       <c r="Q9" s="9" t="inlineStr"/>
+      <c r="R9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1277,6 +1291,11 @@
       <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>Required</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>The mail “Your mutual fund pledge is successful” is currently received once the loan lodgement is successful; it is supposed to come right after the pledging is successful.</t>
         </is>
       </c>
     </row>
@@ -1340,6 +1359,7 @@
       <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr"/>
       <c r="Q11" s="9" t="inlineStr"/>
+      <c r="R11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -1401,6 +1421,7 @@
       <c r="O12" s="7" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr"/>
       <c r="Q12" s="9" t="inlineStr"/>
+      <c r="R12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -1462,6 +1483,7 @@
       <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr"/>
       <c r="Q13" s="9" t="inlineStr"/>
+      <c r="R13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -1523,6 +1545,7 @@
       <c r="O14" s="11" t="inlineStr"/>
       <c r="P14" s="11" t="inlineStr"/>
       <c r="Q14" s="14" t="inlineStr"/>
+      <c r="R14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -1584,6 +1607,7 @@
       <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr"/>
       <c r="Q15" s="9" t="inlineStr"/>
+      <c r="R15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -1645,6 +1669,7 @@
       <c r="O16" s="11" t="inlineStr"/>
       <c r="P16" s="11" t="inlineStr"/>
       <c r="Q16" s="14" t="inlineStr"/>
+      <c r="R16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -1706,6 +1731,7 @@
       <c r="O17" s="11" t="inlineStr"/>
       <c r="P17" s="11" t="inlineStr"/>
       <c r="Q17" s="14" t="inlineStr"/>
+      <c r="R17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -1767,6 +1793,7 @@
       <c r="O18" s="11" t="inlineStr"/>
       <c r="P18" s="11" t="inlineStr"/>
       <c r="Q18" s="14" t="inlineStr"/>
+      <c r="R18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1879,6 +1906,7 @@
           <t>Required</t>
         </is>
       </c>
+      <c r="R19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1995,6 +2023,7 @@
           <t>Required</t>
         </is>
       </c>
+      <c r="R20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2056,6 +2085,7 @@
       <c r="O21" s="3" t="inlineStr"/>
       <c r="P21" s="3" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2164,6 +2194,7 @@
           <t>Required</t>
         </is>
       </c>
+      <c r="R22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -2225,6 +2256,7 @@
       <c r="O23" s="11" t="inlineStr"/>
       <c r="P23" s="11" t="inlineStr"/>
       <c r="Q23" s="14" t="inlineStr"/>
+      <c r="R23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -2286,6 +2318,7 @@
       <c r="O24" s="11" t="inlineStr"/>
       <c r="P24" s="11" t="inlineStr"/>
       <c r="Q24" s="14" t="inlineStr"/>
+      <c r="R24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2390,6 +2423,7 @@
           <t>Required</t>
         </is>
       </c>
+      <c r="R25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2451,6 +2485,7 @@
       <c r="O26" s="3" t="inlineStr"/>
       <c r="P26" s="3" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
+      <c r="R26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -2512,6 +2547,7 @@
       <c r="O27" s="11" t="inlineStr"/>
       <c r="P27" s="11" t="inlineStr"/>
       <c r="Q27" s="14" t="inlineStr"/>
+      <c r="R27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2573,6 +2609,7 @@
       <c r="O28" s="3" t="inlineStr"/>
       <c r="P28" s="3" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2634,6 +2671,7 @@
       <c r="O29" s="3" t="inlineStr"/>
       <c r="P29" s="3" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2695,6 +2733,7 @@
       <c r="O30" s="3" t="inlineStr"/>
       <c r="P30" s="3" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2756,6 +2795,7 @@
       <c r="O31" s="3" t="inlineStr"/>
       <c r="P31" s="3" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2817,6 +2857,7 @@
       <c r="O32" s="3" t="inlineStr"/>
       <c r="P32" s="3" t="inlineStr"/>
       <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2878,6 +2919,7 @@
       <c r="O33" s="3" t="inlineStr"/>
       <c r="P33" s="3" t="inlineStr"/>
       <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2939,6 +2981,7 @@
       <c r="O34" s="3" t="inlineStr"/>
       <c r="P34" s="3" t="inlineStr"/>
       <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3000,6 +3043,7 @@
       <c r="O35" s="3" t="inlineStr"/>
       <c r="P35" s="3" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3061,6 +3105,7 @@
       <c r="O36" s="3" t="inlineStr"/>
       <c r="P36" s="3" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3122,6 +3167,7 @@
       <c r="O37" s="3" t="inlineStr"/>
       <c r="P37" s="3" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3183,6 +3229,7 @@
       <c r="O38" s="3" t="inlineStr"/>
       <c r="P38" s="3" t="inlineStr"/>
       <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3244,6 +3291,7 @@
       <c r="O39" s="3" t="inlineStr"/>
       <c r="P39" s="3" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -3305,6 +3353,7 @@
       <c r="O40" s="11" t="inlineStr"/>
       <c r="P40" s="11" t="inlineStr"/>
       <c r="Q40" s="14" t="inlineStr"/>
+      <c r="R40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3366,6 +3415,7 @@
       <c r="O41" s="3" t="inlineStr"/>
       <c r="P41" s="3" t="inlineStr"/>
       <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3427,6 +3477,7 @@
       <c r="O42" s="3" t="inlineStr"/>
       <c r="P42" s="3" t="inlineStr"/>
       <c r="Q42" s="5" t="inlineStr"/>
+      <c r="R42" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
@@ -3471,7 +3522,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q42"/>
+  <autoFilter ref="A1:R42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>

</xml_diff>

<commit_message>
Communications: remarks for withdrawal-confirmed SMS timing and disbursement No./UTRN format; Loan Disbursed mail with 12-row repayment schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2485,7 +2485,11 @@
       <c r="O26" s="3" t="inlineStr"/>
       <c r="P26" s="3" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
-      <c r="R26" s="3" t="inlineStr"/>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>This SMS has to come once the withdrawal OTP is verified successfully, but it currently comes only once the UTR is approved in the LMS.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -2575,7 +2579,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -2603,13 +2607,107 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr"/>
-      <c r="N28" s="3" t="inlineStr"/>
-      <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="3" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr"/>
-      <c r="R28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Loan Disbursed
+Dear {{CUSTOMER_NAME}},
+We are happy to inform you that your loan amount of ₹{{DISBURSED_AMOUNT}} has been credited to your bank account.
+LOAN DETAILS
+Customer ID: {{CUSTOMER_ID}}
+Loan Account ID: {{LOAN_ACCOUNT_ID}}
+Disbursement Type: {{DISBURSEMENT_TYPE}}
+Disbursement No.: {{DISBURSEMENT_NO}}
+Disbursement UTRN: {{UTRN}}
+Loan Tenure: {{LOAN_TENURE}} months
+EMI Amount: ₹{{EMI_AMOUNT}}
+First EMI Due Date: {{FIRST_EMI_DATE}}
+Balance Amount Available: ₹{{BALANCE_AMOUNT}}
+REPAYMENT SCHEDULE (12 rows – one per month of the 12-month tenure; a 13th row is shown only when required)
+Repayment Date | Repayment Amount
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+DD-MMM-YYYY | ₹XXXXXXX
+(13th row only when required) DD-MMM-YYYY | ₹XXXXXXX
+Please note that the purpose of the loan, as confirmed by you, is {{PURPOSE}} and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Loan Disbursed
+Dear AZHAGARSAMY,
+We are happy to inform you that your loan amount of ₹10,000 has been credited to your bank account.
+LOAN DETAILS
+Customer ID: SCCL1000102
+Loan Account ID: SCCLMF20261000102
+Disbursement Type: Multiple
+Disbursement No.: 1
+Disbursement UTRN: UTIBR52026102700001
+Loan Tenure: 12 months
+EMI Amount: ₹88
+First EMI Due Date: 05-Dec-2026
+Balance Amount Available: ₹1,55,26,100
+REPAYMENT SCHEDULE (12 rows – one per month of the 12-month tenure; a 13th row is shown only when required)
+Repayment Date | Repayment Amount
+05-Dec-2026 | ₹88
+05-Jan-2027 | ₹88
+05-Feb-2027 | ₹88
+05-Mar-2027 | ₹88
+05-Apr-2027 | ₹88
+05-May-2027 | ₹88
+05-Jun-2027 | ₹88
+05-Jul-2027 | ₹88
+05-Aug-2027 | ₹88
+05-Sep-2027 | ₹88
+05-Oct-2027 | ₹88
+05-Nov-2027 | ₹10,088
+(13th row only when required – not needed in this sample)
+Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>In the disbursement mail, Disbursement No. ({{DISBURSEMENT_NO}}) and Disbursement UTRN ({{UTRN}}) currently show a random format; the format of both has to be defined correctly.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -4011,11 +4109,21 @@
 • EMI Amount: ₹[XXXX]
 • First EMI Due Date: [Date]
 • Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
-Repayment Schedule
+Repayment Schedule – 12 rows, one per month of the 12-month tenure; a 13th row is shown only when required
 Repayment Date | Repayment Amount
 DD-MMM-YYYY | ₹XXXXXX
 DD-MMM-YYYY | ₹XXXXXX
 DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+(13th row only when required) DD-MMM-YYYY | ₹XXXXXX
 Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
 Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
 Warm regards,
@@ -4038,11 +4146,21 @@
 • EMI Amount: ₹88
 • First EMI Due Date: 05-11-2026
 • Balance amount available ₹1,55,26,100 (If disbursement type is MULTIPLE.)
-Repayment Schedule
+Repayment Schedule – 12 rows, one per month of the 12-month tenure; a 13th row is shown only when required
 Repayment Date | Repayment Amount
 DD-MMM-YYYY | ₹XXXXXX
 DD-MMM-YYYY | ₹XXXXXX
 DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+DD-MMM-YYYY | ₹XXXXXX
+(13th row only when required) DD-MMM-YYYY | ₹XXXXXX
 Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
 Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
 Warm regards,

</xml_diff>

<commit_message>
Communications: EMI reminder row now SMS + Mail (T-5 template); mail reader handles table rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2735,7 +2735,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2763,12 +2763,63 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="3" t="inlineStr"/>
-      <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="3" t="inlineStr"/>
-      <c r="Q29" s="5" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Reminder: Your EMI of ₹{{EMI_AMOUNT}} is due on {{DUE_DATE}}</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Reminder: Your EMI of ₹10,000 is due on 05-11-2026</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 5 days before the original EMI presentation date (T-5)
+EMI Due Reminder
+Dear {{CUSTOMER_NAME}},
+This is a friendly reminder that your next EMI of ₹{{EMI_AMOUNT}} for your loan will be automatically deducted from your bank account on {{DUE_DATE}}. Kindly ensure that your account has sufficient funds to cover the payment.
+Loan Details
+Borrowed Amount: ₹{{BORROWED_AMOUNT}}
+Outstanding Amount: ₹{{OUTSTANDING_AMOUNT}}
+Bank Account Number: {{BANK_ACCOUNT_NUMBER}}
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to ensure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 5 days before the original EMI presentation date (T-5)
+EMI Due Reminder
+Dear AZHAGARSAMY,
+This is a friendly reminder that your next EMI of ₹10,000 for your loan will be automatically deducted from your bank account on 05-11-2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Loan Details
+Borrowed Amount: ₹1,00,000
+Outstanding Amount: ₹1,00,000
+Bank Account Number: XXXXXXXX8736
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to ensure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
@@ -3628,6 +3679,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: EMI Reminder (T-5) scenario clarified (1st of every month); EMI Presentation Reminder (T-1) mail-only row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2715,12 +2715,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>EMI Reminder</t>
+          <t>EMI Reminder (T-5)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer of an upcoming instalment before its due date</t>
+          <t>First EMI reminder: sent on the 1st of every month – T-5 / T-4 before the EMI presentation date – notifying the customer of the upcoming instalment (SMS and mail). The second reminder, T-1, is mail only (next row)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>Trigger: 5 days before the original EMI presentation date (T-5)
+          <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
 EMI Due Reminder
 Dear {{CUSTOMER_NAME}},
 This is a friendly reminder that your next EMI of ₹{{EMI_AMOUNT}} for your loan will be automatically deducted from your bank account on {{DUE_DATE}}. Kindly ensure that your account has sufficient funds to cover the payment.
@@ -2793,7 +2793,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Trigger: 5 days before the original EMI presentation date (T-5)
+          <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
 EMI Due Reminder
 Dear AZHAGARSAMY,
 This is a friendly reminder that your next EMI of ₹10,000 for your loan will be automatically deducted from your bank account on 05-11-2026. Kindly ensure that your account has sufficient funds to cover the payment.
@@ -2828,12 +2828,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>EMI Success</t>
+          <t>EMI Presentation Reminder (T-1)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment is debited successfully</t>
+          <t>Second EMI reminder: sent 1 day before the EMI presentation date (T-1) – mail only, no SMS. The first reminder, T-5, is the row above</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2848,40 +2848,91 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>Mail</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>SGRCDT-T</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>EMI Presentation Alert – {{DATE}}</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>EMI Presentation Alert – 05-11-2026</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 1 day before the EMI presentation date (T-1)
+EMI Presentation Alert
+Dear {{CUSTOMER_NAME}},
+This is a reminder that your next EMI of ₹{{EMI_AMOUNT}} for your loan will be automatically deducted from your bank account on {{DATE}}. Kindly ensure that your account has sufficient funds to cover the payment.
+Loan Details
+Borrowed Amount: ₹{{BORROWED_AMOUNT}}
+Outstanding Amount: ₹{{OUTSTANDING_AMOUNT}}
+Bank Account Number: {{BANK_ACCOUNT_NUMBER}}
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to ensure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 1 day before the EMI presentation date (T-1)
+EMI Presentation Alert
+Dear AZHAGARSAMY,
+This is a reminder that your next EMI of ₹10,000 for your loan will be automatically deducted from your bank account on 05-11-2026. Kindly ensure that your account has sufficient funds to cover the payment.
+Loan Details
+Borrowed Amount: ₹1,00,000
+Outstanding Amount: ₹1,00,000
+Bank Account Number: XXXXXXXX8736
+Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to ensure that your account balance is adequate to avoid any inconvenience.
+Thank you for your cooperation.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
-      <c r="N30" s="3" t="inlineStr"/>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr"/>
-      <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
@@ -2890,12 +2941,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>EMI Failed</t>
+          <t>EMI Success</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+          <t>Notifying the customer when the instalment is debited successfully</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2915,12 +2966,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2952,12 +3003,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Reminder</t>
+          <t>EMI Failed</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2977,12 +3028,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -3014,12 +3065,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Success</t>
+          <t>EMI Resubmission Reminder</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission is successful</t>
+          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -3039,12 +3090,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3076,12 +3127,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Failed</t>
+          <t>EMI Resubmission Success</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+          <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -3101,12 +3152,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3138,12 +3189,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>LAMF Part Payment Confirmation</t>
+          <t>EMI Resubmission Failed</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -3163,12 +3214,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -3200,12 +3251,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>LTV Breach Trigger (Margin Call)</t>
+          <t>LAMF Part Payment Confirmation</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
+          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3225,12 +3276,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -3262,12 +3313,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>LAMF LTV Breach Liquidation</t>
+          <t>LTV Breach Trigger (Margin Call)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -3287,12 +3338,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -3324,12 +3375,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>LAMF Principal Repayment Reminder</t>
+          <t>LAMF LTV Breach Liquidation</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -3349,12 +3400,12 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -3386,12 +3437,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>LAMF Liquidation for O/S</t>
+          <t>LAMF Principal Repayment Reminder</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3411,12 +3462,12 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -3443,128 +3494,128 @@
       <c r="R39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n">
+      <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Liquidation for O/S</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr"/>
+      <c r="N40" s="3" t="inlineStr"/>
+      <c r="O40" s="3" t="inlineStr"/>
+      <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Foreclosure Completed</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E40" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G40" s="11" t="inlineStr">
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr">
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I40" s="12" t="inlineStr">
+      <c r="I41" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J40" s="13" t="inlineStr">
+      <c r="J41" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K40" s="11" t="inlineStr">
+      <c r="K41" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="L40" s="11" t="inlineStr"/>
-      <c r="M40" s="11" t="inlineStr"/>
-      <c r="N40" s="11" t="inlineStr"/>
-      <c r="O40" s="11" t="inlineStr"/>
-      <c r="P40" s="11" t="inlineStr"/>
-      <c r="Q40" s="14" t="inlineStr"/>
-      <c r="R40" s="11" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Successful Loan Tenure Completion</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr"/>
-      <c r="O41" s="3" t="inlineStr"/>
-      <c r="P41" s="3" t="inlineStr"/>
-      <c r="Q41" s="5" t="inlineStr"/>
-      <c r="R41" s="3" t="inlineStr"/>
+      <c r="L41" s="11" t="inlineStr"/>
+      <c r="M41" s="11" t="inlineStr"/>
+      <c r="N41" s="11" t="inlineStr"/>
+      <c r="O41" s="11" t="inlineStr"/>
+      <c r="P41" s="11" t="inlineStr"/>
+      <c r="Q41" s="14" t="inlineStr"/>
+      <c r="R41" s="11" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3572,12 +3623,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Loan Account Closure</t>
+          <t>Successful Loan Tenure Completion</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>When the loan account is closed (closed on = loan end date)</t>
+          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3597,12 +3648,12 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -3628,50 +3679,112 @@
       <c r="Q42" s="5" t="inlineStr"/>
       <c r="R42" s="3" t="inlineStr"/>
     </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Loan Account Closure</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>When the loan account is closed (closed on = loan end date)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr"/>
+      <c r="N43" s="3" t="inlineStr"/>
+      <c r="O43" s="3" t="inlineStr"/>
+      <c r="P43" s="3" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="R43" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
+          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
+          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
+          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R42"/>
+  <autoFilter ref="A1:R43"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>
@@ -3680,6 +3793,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Loan Disbursed split into First Disbursement (SMS+mail) and Subsequent Disbursement (mail only, 08 template)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2559,12 +2559,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Loan Disbursed</t>
+          <t>Loan Disbursed (First Disbursement)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>When the loan is disbursed – notifying the customer that the amount is credited to the bank account</t>
+          <t>When the loan is disbursed for the first time (first disbursement) – notifying the customer that the amount is credited to the bank account. Each subsequent withdrawal is the mail-only row below</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2715,65 +2715,202 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
+          <t>Loan Disbursed (Subsequent Disbursement)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>On each subsequent withdrawal / disbursement after the first one – notifying the customer that the amount is credited to the bank account (mail only, no SMS). The first disbursement is the row above</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Loan disbursed to your account</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
+Loan Disbursed
+Dear {{CUSTOMER_NAME}},
+We are happy to inform you that your loan amount of ₹{{LOAN_AMOUNT}} has been credited to your bank account.
+Loan Details
+Customer ID: {{CUSTOMER_ID}}
+Loan Account ID: {{LOAN_ACCOUNT_ID}}
+Disbursement Type: Multiple
+Disbursement No.: {{DISBURSEMENT_NO}}
+Disbursement UTRN: {{UTRN}}
+Loan Tenure: {{LOAN_TENURE}} months
+EMI Amount (this disbursement, 30-day cycle): ₹{{EMI_AMOUNT}}
+First EMI Due Date: {{FIRST_EMI_DATE}}
+Balance Amount Available: ₹{{BALANCE_AMOUNT}}
+Repayment Schedule
+Cumulative of all disbursements to date — residual term shown
+Repayment Date: Repayment Amount
+DD-MMM-YYYY: ₹XXXXXX
+DD-MMM-YYYY: ₹XXXXXX
+DD-MMM-YYYY: ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is {{PURPOSE}} and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
+Loan Disbursed
+Dear AZHAGARSAMY,
+We are happy to inform you that your loan amount of ₹20,000 has been credited to your bank account.
+Loan Details
+Customer ID: SCCL1000102
+Loan Account ID: SCCLMF20261000102
+Disbursement Type: Multiple
+Disbursement No.: 2
+Disbursement UTRN: UTIBR52026110200002
+Loan Tenure: 12 months
+EMI Amount (this disbursement, 30-day cycle): ₹175
+First EMI Due Date: 05-Dec-2026
+Balance Amount Available: ₹1,55,06,100
+Repayment Schedule
+Cumulative of all disbursements to date — residual term shown
+Repayment Date: Repayment Amount
+DD-MMM-YYYY: ₹XXXXXX
+DD-MMM-YYYY: ₹XXXXXX
+DD-MMM-YYYY: ₹XXXXXX
+Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
           <t>EMI Reminder (T-5)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>First EMI reminder: sent on the 1st of every month – T-5 / T-4 before the EMI presentation date – notifying the customer of the upcoming instalment (SMS and mail). The second reminder, T-1, is mail only (next row)</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>Reminder: Your EMI of ₹{{EMI_AMOUNT}} is due on {{DUE_DATE}}</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>Reminder: Your EMI of ₹10,000 is due on 05-11-2026</t>
         </is>
       </c>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
 EMI Due Reminder
@@ -2791,7 +2928,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
 EMI Due Reminder
@@ -2809,84 +2946,84 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="R29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="R30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>EMI Presentation Reminder (T-1)</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Second EMI reminder: sent 1 day before the EMI presentation date (T-1) – mail only, no SMS. The first reminder, T-5, is the row above</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Mail</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – {{DATE}}</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – 05-11-2026</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2904,7 +3041,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2922,79 +3059,17 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="P31" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
+      <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="R30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>EMI Success</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Notifying the customer when the instalment is debited successfully</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr"/>
-      <c r="N31" s="3" t="inlineStr"/>
-      <c r="O31" s="3" t="inlineStr"/>
-      <c r="P31" s="3" t="inlineStr"/>
-      <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
@@ -3003,12 +3078,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>EMI Failed</t>
+          <t>EMI Success</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+          <t>Notifying the customer when the instalment is debited successfully</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -3028,12 +3103,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -3065,12 +3140,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Reminder</t>
+          <t>EMI Failed</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
+          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -3090,12 +3165,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3127,12 +3202,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Success</t>
+          <t>EMI Resubmission Reminder</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission is successful</t>
+          <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -3152,12 +3227,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3189,12 +3264,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>EMI Resubmission Failed</t>
+          <t>EMI Resubmission Success</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
+          <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -3214,12 +3289,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -3251,12 +3326,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>LAMF Part Payment Confirmation</t>
+          <t>EMI Resubmission Failed</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
+          <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3276,12 +3351,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -3313,12 +3388,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>LTV Breach Trigger (Margin Call)</t>
+          <t>LAMF Part Payment Confirmation</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
+          <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -3338,12 +3413,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -3375,12 +3450,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>LAMF LTV Breach Liquidation</t>
+          <t>LTV Breach Trigger (Margin Call)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
+          <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -3400,12 +3475,12 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -3437,12 +3512,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>LAMF Principal Repayment Reminder</t>
+          <t>LAMF LTV Breach Liquidation</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
+          <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3462,12 +3537,12 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -3499,12 +3574,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>LAMF Liquidation for O/S</t>
+          <t>LAMF Principal Repayment Reminder</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+          <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -3524,12 +3599,12 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -3556,128 +3631,128 @@
       <c r="R40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="n">
+      <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>LAMF Liquidation for O/S</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr"/>
+      <c r="N41" s="3" t="inlineStr"/>
+      <c r="O41" s="3" t="inlineStr"/>
+      <c r="P41" s="3" t="inlineStr"/>
+      <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Foreclosure Completed</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F41" s="11" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
+      <c r="G42" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr">
+      <c r="H42" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I41" s="12" t="inlineStr">
+      <c r="I42" s="12" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J41" s="13" t="inlineStr">
+      <c r="J42" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K41" s="11" t="inlineStr">
+      <c r="K42" s="11" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="L41" s="11" t="inlineStr"/>
-      <c r="M41" s="11" t="inlineStr"/>
-      <c r="N41" s="11" t="inlineStr"/>
-      <c r="O41" s="11" t="inlineStr"/>
-      <c r="P41" s="11" t="inlineStr"/>
-      <c r="Q41" s="14" t="inlineStr"/>
-      <c r="R41" s="11" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Successful Loan Tenure Completion</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>SGRCDT-T</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L42" s="3" t="inlineStr"/>
-      <c r="M42" s="3" t="inlineStr"/>
-      <c r="N42" s="3" t="inlineStr"/>
-      <c r="O42" s="3" t="inlineStr"/>
-      <c r="P42" s="3" t="inlineStr"/>
-      <c r="Q42" s="5" t="inlineStr"/>
-      <c r="R42" s="3" t="inlineStr"/>
+      <c r="L42" s="11" t="inlineStr"/>
+      <c r="M42" s="11" t="inlineStr"/>
+      <c r="N42" s="11" t="inlineStr"/>
+      <c r="O42" s="11" t="inlineStr"/>
+      <c r="P42" s="11" t="inlineStr"/>
+      <c r="Q42" s="14" t="inlineStr"/>
+      <c r="R42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3685,12 +3760,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Loan Account Closure</t>
+          <t>Successful Loan Tenure Completion</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>When the loan account is closed (closed on = loan end date)</t>
+          <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3710,12 +3785,12 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+          <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -3741,50 +3816,112 @@
       <c r="Q43" s="5" t="inlineStr"/>
       <c r="R43" s="3" t="inlineStr"/>
     </row>
-    <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Loan Account Closure</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>When the loan account is closed (closed on = loan end date)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>SCCL</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr"/>
+      <c r="O44" s="3" t="inlineStr"/>
+      <c r="P44" s="3" t="inlineStr"/>
+      <c r="Q44" s="5" t="inlineStr"/>
+      <c r="R44" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
+          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
+          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
+          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R43"/>
+  <autoFilter ref="A1:R44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId2"/>
@@ -3794,6 +3931,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: EMI Failed (bounce on the 5th) gets the Bounce - 1A mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3145,7 +3145,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Notifying the customer when the instalment bounces (rejected by the bank); the debit is retried on the 10th</t>
+          <t>Notifying the customer when the instalment presented on the 5th of the month bounces (rejected by the bank); the debit is retried on the 10th – SMS and mail</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -3188,12 +3188,57 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="3" t="inlineStr"/>
-      <c r="O33" s="3" t="inlineStr"/>
-      <c r="P33" s="3" t="inlineStr"/>
-      <c r="Q33" s="5" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Alert: Your EMI payment failed {{LOAN_ID}}</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Alert: Your EMI payment failed SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
+Instalment Failure / EMI Bounce Notification (Bounce - 1A)
+Dear {{CUSTOMER_NAME}},
+We could not process your EMI of ₹{{EMI_AMOUNT}} for the loan account {{LOAN_ID}} on {{BOUNCE_DATE}} due to insufficient balance.
+We will re-present the EMI on {{REPRESENTATION_DATE}}. Please ensure your account has a sufficient balance to avoid penalties.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
+Instalment Failure / EMI Bounce Notification (Bounce - 1A)
+Dear AZHAGARSAMY,
+We could not process your EMI of ₹10,000 for the loan account SCCLMF20261000102 on 05-11-2026 due to insufficient balance.
+We will re-present the EMI on 10-11-2026. Please ensure your account has a sufficient balance to avoid penalties.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
@@ -3932,6 +3977,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: EMI Success gets the Successful EMI Deduction mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -3126,12 +3126,65 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr"/>
-      <c r="N32" s="3" t="inlineStr"/>
-      <c r="O32" s="3" t="inlineStr"/>
-      <c r="P32" s="3" t="inlineStr"/>
-      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Your EMI of ₹{{EMI_AMOUNT}} Has Been Successfully Deducted</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Your EMI of ₹10,000 Has Been Successfully Deducted</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>EMI Payment Confirmed
+Dear {{CUSTOMER_NAME}},
+We are writing to confirm that your EMI of ₹{{EMI_AMOUNT}} for the loan account {{LOAN_ID}} was successfully debited on {{DEDUCTION_DATE}} from your registered bank account.
+✓ EMI Successfully Deducted
+EMI Details
+Loan Account Number: {{LOAN_ID}}
+EMI Amount: ₹{{EMI_AMOUNT}}
+Deduction Date: {{DEDUCTION_DATE}}
+Next EMI Due Date: {{NEXT_EMI_DATE}}
+Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>EMI Payment Confirmed
+Dear AZHAGARSAMY,
+We are writing to confirm that your EMI of ₹10,000 for the loan account SCCLMF20261000102 was successfully debited on 05-11-2026 from your registered bank account.
+✓ EMI Successfully Deducted
+EMI Details
+Loan Account Number: SCCLMF20261000102
+EMI Amount: ₹10,000
+Deduction Date: 05-11-2026
+Next EMI Due Date: 05-12-2026
+Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
@@ -3977,7 +4030,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: remark on EMI Failed – mail title to be EMI Payment Failed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3292,7 +3292,11 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>In the mail, the title “Instalment Failure / EMI Bounce Notification (Bounce - 1A)” has to be changed to “EMI Payment Failed”.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">

</xml_diff>

<commit_message>
Communications: remark on EMI Success – Next EMI Due Date for the last EMI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3185,7 +3185,11 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="R32" s="3" t="inlineStr"/>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>In the mail, “Next EMI Due Date: {{NEXT_EMI_DATE}}” – what is shown for the last EMI (12th EMI), when there is no next EMI, has to be defined.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">

</xml_diff>

<commit_message>
Communications: Part Payment Confirmation gets the Part Payment mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3514,7 +3514,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -3542,12 +3542,65 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr"/>
-      <c r="N37" s="3" t="inlineStr"/>
-      <c r="O37" s="3" t="inlineStr"/>
-      <c r="P37" s="3" t="inlineStr"/>
-      <c r="Q37" s="5" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Attachment: Updated Repayment Schedule PDF
+Part Payment Processed
+Dear {{CUSTOMER_NAME}},
+We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
+Payment Summary
+Transaction Status: ✓ Successful
+Amount Received: ₹{{AMOUNT_RECEIVED}}
+Revised Outstanding Balance: ₹{{REVISED_OUTSTANDING_BALANCE}}
+📄 Updated Repayment Schedule attached. As a result of this payment, your repayment schedule has been revised — please review the attached document for the latest schedule.
+Should you have any questions, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Attachment: Updated Repayment Schedule PDF
+Part Payment Processed
+Dear AZHAGARSAMY,
+We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
+Payment Summary
+Transaction Status: ✓ Successful
+Amount Received: ₹5,000
+Revised Outstanding Balance: ₹5,000
+📄 Updated Repayment Schedule attached. As a result of this payment, your repayment schedule has been revised — please review the attached document for the latest schedule.
+Should you have any questions, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -4040,6 +4093,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Foreclosure Completed gets the Pre-Closure mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3877,7 +3877,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
@@ -3905,12 +3905,75 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L42" s="11" t="inlineStr"/>
-      <c r="M42" s="11" t="inlineStr"/>
-      <c r="N42" s="11" t="inlineStr"/>
-      <c r="O42" s="11" t="inlineStr"/>
-      <c r="P42" s="11" t="inlineStr"/>
-      <c r="Q42" s="14" t="inlineStr"/>
+      <c r="L42" s="11" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
+        </is>
+      </c>
+      <c r="M42" s="11" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
+        </is>
+      </c>
+      <c r="N42" s="11" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation
+Dear {{CUSTOMER_NAME}},
+✓ Loan Successfully Pre-Closed
+Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit. We have received the final payment and are pleased to confirm that your loan account has been closed in our records.
+We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process
+Status: Lien release process initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a separate notification from CAMS/KFintech once units are fully unlocked.
+Next Steps
+📄 No Objection Certificate (NOC): Your formal NOC is being generated and will be sent to you in a separate communication shortly.
+Important Information
+• Please retain this email as confirmation of loan closure until you receive your formal NOC.
+• If the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, please reach out to our customer support at lassupport@shriramcredit.in.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O42" s="11" t="inlineStr">
+        <is>
+          <t>Loan Pre-Closure Confirmation
+Dear AZHAGARSAMY,
+✓ Loan Successfully Pre-Closed
+Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit. We have received the final payment and are pleased to confirm that your loan account has been closed in our records.
+We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process
+Status: Lien release process initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a separate notification from CAMS/KFintech once units are fully unlocked.
+Next Steps
+📄 No Objection Certificate (NOC): Your formal NOC is being generated and will be sent to you in a separate communication shortly.
+Important Information
+• Please retain this email as confirmation of loan closure until you receive your formal NOC.
+• If the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, please reach out to our customer support at lassupport@shriramcredit.in.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P42" s="11" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q42" s="13" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
@@ -4094,6 +4157,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Loan Tenure Completion gets the closure mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -4002,7 +4002,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -4030,12 +4030,77 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L43" s="3" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr"/>
-      <c r="N43" s="3" t="inlineStr"/>
-      <c r="O43" s="3" t="inlineStr"/>
-      <c r="P43" s="3" t="inlineStr"/>
-      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Congratulations on completing your loan journey</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>Congratulations on completing your loan journey</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
+Loan Journey Complete
+Dear {{CUSTOMER_NAME}},
+✓ Congratulations on Completing Your Loan Journey!
+Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit. We have received the final payment and are pleased to confirm that your loan account has been closed in our records.
+We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process
+Status: Lien release process initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a notification from CAMS/KFintech once your units are fully unlocked.
+Next Steps
+📄 No Objection Certificate (NOC): Your formal NOC is being generated and will be sent to you in a separate communication shortly.
+Important Information
+• Please retain this email as confirmation of loan closure until you receive your formal NOC.
+• If the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, please reach out to our customer support at lassupport@shriramcredit.in.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
+Loan Journey Complete
+Dear AZHAGARSAMY,
+✓ Congratulations on Completing Your Loan Journey!
+Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit. We have received the final payment and are pleased to confirm that your loan account has been closed in our records.
+We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
+Lien Removal Process
+Status: Lien release process initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a notification from CAMS/KFintech once your units are fully unlocked.
+Next Steps
+📄 No Objection Certificate (NOC): Your formal NOC is being generated and will be sent to you in a separate communication shortly.
+Important Information
+• Please retain this email as confirmation of loan closure until you receive your formal NOC.
+• If the lien is not removed within the stated timeline, please contact us for assistance.
+Should you have any questions, please reach out to our customer support at lassupport@shriramcredit.in.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
@@ -4158,6 +4223,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Margin Call gets the MF value drop mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3629,7 +3629,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -3657,12 +3657,61 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
-      <c r="N38" s="3" t="inlineStr"/>
-      <c r="O38" s="3" t="inlineStr"/>
-      <c r="P38" s="3" t="inlineStr"/>
-      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Mutual Fund Margin Shortfall &lt;&lt;Loan ID&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Mutual Fund Margin Shortfall SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: LTV breach – notifying the customer of a margin shortfall
+Margin Call / Mutual Fund Value Drop
+Dear {{CUSTOMER_NAME}},
+⚠ The current market value of your Mutual Fund units pledged with us has declined and current LTV is at {{CURRENT_LTV}}%.
+We request you to make an immediate payment of ₹{{MINIMUM_AMOUNT}} (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of ₹({{SHORTFALL_AMOUNT}}/0.65) or For Debt MF of ₹({{SHORTFALL_AMOUNT}}/0.75)) to bring your account within the prescribed limit.
+Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
+Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
+Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your prompt attention to this matter.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as this mailbox is not monitored and you will not receive a response. Loan Against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: LTV breach – notifying the customer of a margin shortfall
+Margin Call / Mutual Fund Value Drop
+Dear AZHAGARSAMY,
+⚠ The current market value of your Mutual Fund units pledged with us has declined and current LTV is at 82.50%.
+We request you to make an immediate payment of ₹10,000 (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of ₹15,385 or For Debt MF of ₹13,333) to bring your account within the prescribed limit.
+Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
+Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
+Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your prompt attention to this matter.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as this mailbox is not monitored and you will not receive a response. Loan Against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
@@ -4222,8 +4271,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: LTV Breach Liquidation gets the LTV breach beyond policy norms mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3740,7 +3740,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -3768,12 +3768,57 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="3" t="inlineStr"/>
-      <c r="O39" s="3" t="inlineStr"/>
-      <c r="P39" s="3" t="inlineStr"/>
-      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach {{LOAN_ID}}</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>LTV Breach – Liquidation of Pledged Units
+Dear {{CUSTOMER_NAME}},
+⚠ Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of Loan Agreement.
+Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>LTV Breach – Liquidation of Pledged Units
+Dear AZHAGARSAMY,
+⚠ Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of Loan Agreement.
+Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
@@ -4272,8 +4317,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Loan Account Closure gets the NOC / Loan Closure Certificate mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -4223,7 +4223,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -4251,12 +4251,61 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L44" s="3" t="inlineStr"/>
-      <c r="M44" s="3" t="inlineStr"/>
-      <c r="N44" s="3" t="inlineStr"/>
-      <c r="O44" s="3" t="inlineStr"/>
-      <c r="P44" s="3" t="inlineStr"/>
-      <c r="Q44" s="5" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Your Loan Account {{LOAN_ID}} is closed successfully</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>Your Loan Account SCCLMF20261000102 is closed successfully</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: manual trigger
+Attachment: NOC / Loan Closure Certificate PDF
+No Objection Certificate
+Dear {{CUSTOMER_NAME}},
+✓ Loan Account Closed Successfully
+We are pleased to inform you that your loan account {{LOAN_ID}} has been closed successfully.
+📄 No Objection Certificate (NOC) is attached to this email for your records. Please retain it as formal confirmation of loan closure.
+Your Customer ID remains active with us, and you are always welcome to visit us for any future financial requirements.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: manual trigger
+Attachment: NOC / Loan Closure Certificate PDF
+No Objection Certificate
+Dear AZHAGARSAMY,
+✓ Loan Account Closed Successfully
+We are pleased to inform you that your loan account SCCLMF20261000102 has been closed successfully.
+📄 No Objection Certificate (NOC) is attached to this email for your records. Please retain it as formal confirmation of loan closure.
+Your Customer ID remains active with us, and you are always welcome to visit us for any future financial requirements.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is only for personal use. The loan amount cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R44" s="3" t="inlineStr"/>
     </row>
     <row r="46">
@@ -4320,6 +4369,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Liquidation for O/S gets the Liquidation for Outstanding Loan mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3909,7 +3909,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -3937,12 +3937,57 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr"/>
-      <c r="O41" s="3" t="inlineStr"/>
-      <c r="P41" s="3" t="inlineStr"/>
-      <c r="Q41" s="5" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan {{LOAN_ID}}</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Liquidation for Outstanding Loan
+Dear {{CUSTOMER_NAME}},
+The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of Loan Agreement.
+Any surplus amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>Liquidation for Outstanding Loan
+Dear AZHAGARSAMY,
+The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
+Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of Loan Agreement.
+Any surplus amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
+Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
+Thank you for your understanding.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
@@ -4367,9 +4412,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: Principal Repayment Reminder gets the Principal Repayment for Loan Closure mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3847,7 +3847,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -3875,12 +3875,67 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="3" t="inlineStr"/>
-      <c r="O40" s="3" t="inlineStr"/>
-      <c r="P40" s="3" t="inlineStr"/>
-      <c r="Q40" s="5" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Principal Repayment {{LOAN_ID}}</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Action Required: Principal Repayment SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>Principal Repayment for Loan Closure
+Dear {{CUSTOMER_NAME}},
+⚠ Notice: Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
+As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
+Please note that:
+• Interest at the applicable contractual rate shall continue to accrue during the grace period.
+• The outstanding amount must be repaid within the stipulated grace period.
+Please use the below link to check the details and make payment.
+[Make Payment →]
+Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of Loan Agreement.
+Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
+Thank you for your prompt attention.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>Principal Repayment for Loan Closure
+Dear AZHAGARSAMY,
+⚠ Notice: Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
+As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
+Please note that:
+• Interest at the applicable contractual rate shall continue to accrue during the grace period.
+• The outstanding amount must be repaid within the stipulated grace period.
+Please use the below link to check the details and make payment.
+[Make Payment →]
+Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of Loan Agreement.
+Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
+Thank you for your prompt attention.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
@@ -4412,10 +4467,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: EMI Resubmission Reminder gets the 1B T-1 mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3328,7 +3328,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -3356,12 +3356,55 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr"/>
-      <c r="N34" s="3" t="inlineStr"/>
-      <c r="O34" s="3" t="inlineStr"/>
-      <c r="P34" s="3" t="inlineStr"/>
-      <c r="Q34" s="5" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Final Reminder: EMI Re-presentation on {{REPRESENTATION_DATE}} &lt;&lt;{{LOAN_ID}}&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Final Reminder: EMI Re-presentation on 10-11-2026 SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
+Second EMI Representation Reminder (1B T-1)
+Dear {{CUSTOMER_NAME}},
+This is to inform you that your EMI of ₹{{EMI_AMOUNT}} will be re-presented on {{REPRESENTATION_DATE}}.
+⚠ Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
+Second EMI Representation Reminder (1B T-1)
+Dear AZHAGARSAMY,
+This is to inform you that your EMI of ₹10,000 will be re-presented on 10-11-2026.
+⚠ Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
+In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
@@ -4464,14 +4507,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: EMI Resubmission Failed gets the 2B Bounce mail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3495,7 +3495,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -3523,12 +3523,51 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr"/>
-      <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr"/>
-      <c r="P36" s="3" t="inlineStr"/>
-      <c r="Q36" s="5" t="inlineStr"/>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Urgent: Mutual Fund Liquidation Scheduled {{LOAN_ID}}</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>Urgent: Mutual Fund Liquidation Scheduled SCCLMF20261000102</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Initiation of Loan Closure Procedures (2B Bounce)
+Dear {{CUSTOMER_NAME}},
+Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Initiation of Loan Closure Procedures (2B Bounce)
+Dear AZHAGARSAMY,
+Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer: This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.
+© 2026 Shriram Credit Company Limited. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>Yes
+View mail</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="R36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
@@ -4508,14 +4547,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: subsequent disbursement sends the same SMS as the first disbursement
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>When the loan is disbursed for the first time (first disbursement) – notifying the customer that the amount is credited to the bank account. Each subsequent withdrawal is the mail-only row below</t>
+          <t>When the loan is disbursed for the first time (first disbursement) – notifying the customer that the amount is credited to the bank account. Each subsequent withdrawal is the row below (same SMS, different mail)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>On each subsequent withdrawal / disbursement after the first one – notifying the customer that the amount is credited to the bank account (mail only, no SMS). The first disbursement is the row above</t>
+          <t>On each subsequent withdrawal / disbursement after the first one – notifying the customer that the amount is credited to the bank account. Same SMS as the first disbursement (row above); only the mail is different</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2735,32 +2735,32 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Mail</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SGRCDT-T</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Communications: EMI Reminder mail – trigger line removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2912,8 +2912,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
-EMI Due Reminder
+          <t>EMI Due Reminder
 Dear {{CUSTOMER_NAME}},
 This is a friendly reminder that your next EMI of ₹{{EMI_AMOUNT}} for your loan will be automatically deducted from your bank account on {{DUE_DATE}}. Kindly ensure that your account has sufficient funds to cover the payment.
 Loan Details
@@ -2930,8 +2929,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Trigger: 1st of every month – T-5 / T-4 before the EMI presentation date
-EMI Due Reminder
+          <t>EMI Due Reminder
 Dear AZHAGARSAMY,
 This is a friendly reminder that your next EMI of ₹10,000 for your loan will be automatically deducted from your bank account on 05-11-2026. Kindly ensure that your account has sufficient funds to cover the payment.
 Loan Details

</xml_diff>

<commit_message>
Communications: row 29 renamed EMI Presentation Reminder (T-5), scenario reworded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2852,12 +2852,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>EMI Reminder (T-5)</t>
+          <t>EMI Presentation Reminder (T-5)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>First EMI reminder: the EMI is due on the 5th of every month, so this reminder has to be sent on the 1st of every month – notifying the customer of the upcoming instalment (SMS and mail). The second reminder, T-1, is mail only (next row)</t>
+          <t>This communication has to be triggered on the 1st of every month when the EMI is due on the 5th – first reminder of the upcoming instalment (SMS and mail). The second reminder, T-1, is mail only (next row)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Communications: row 30 T-1 reminder – scenario reworded, SMS drafted (to be created)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2958,70 +2958,70 @@
       <c r="R30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>EMI Presentation Reminder (T-1)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Second EMI reminder: sent 1 day before the EMI presentation date (T-1) – mail only, no SMS. The first reminder, T-5, is the row above</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Second EMI reminder: this communication has to be triggered 1 day before the EMI presentation date (T-1), i.e. on the 4th when the EMI is due on the 5th – SMS and mail. SMS template drafted by Claude for approval; to be created and registered. The first reminder, T-5, is the row above</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>SMS, Mail</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} for loan account {#alphanumeric#} will be presented tomorrow, {#alphanumeric#}. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 for loan account SCCLMF20261000102 will be presented tomorrow, 05-11-2026. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>SGRCDT-T</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – {{DATE}}</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="M31" s="11" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – 05-11-2026</t>
         </is>
       </c>
-      <c r="N31" s="3" t="inlineStr">
+      <c r="N31" s="11" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -3039,7 +3039,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="O31" s="11" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -3057,18 +3057,18 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="P31" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q31" s="13" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="R31" s="3" t="inlineStr"/>
+      <c r="R31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">

</xml_diff>

<commit_message>
Communications: separate Mail table and Mail sheet removed; one combined SMS and mail table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -7,12 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMS and Mail" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS'!$A$1:$R$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mail'!$A$1:$K$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS and Mail'!$A$1:$R$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4558,1777 +4556,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
-    <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>S.No</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Scenarios</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Application</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Sender</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Communication Type</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Body (template)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Body (sample)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Mail Subject</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SMS Header</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Email Verification</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>When the customer clicks Verify for the email on the KYC Verification page</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dear Customer,
-XXXXXX is the OTP to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
-Please do not share the OTP with anyone.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Dear Customer,
-123456 is the OTP to verify your email and continue with your Shriram Credit’s Loan Against Mutual Fund application.
-Please do not share the OTP with anyone.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Mutual Fund Pledge Successful</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>After the mutual fund units are successfully pledged</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
-You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Congratulations! Your mutual fund has been successfully pledged against your applied loan with Shriram Credit.
-You are one step closer to receiving your funds. We’ll notify you once the loan is disbursed.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Your mutual fund pledge is successful</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Loan Sanction Letter Mail</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>After the Sanction Letter is generated. To: customer e-mail ID; CC: loandocuments@shriramcredit.in; Sanction Letter attached</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
-For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
-We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved.
-For your reference, we have attached the Loan Sanction Letter, which contains the complete details of your approved loan, including the sanctioned amount, tenure, repayment schedule, interest rate, and applicable terms and conditions.
-We encourage you to review this document thoroughly to ensure you are familiar with the loan structure and repayment obligations.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Loan Agreement Mail</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>After the loan agreement is e-signed. To: customer e-mail ID; CC: loandocuments@shriramcredit.in; signed Loan Agreement attached</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>LOS</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
-Your Loan ID is XXXXXXXX
-📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
-✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been approved, and your loan agreement is now ready for your review.
-Your Loan ID is SCCLMF20261000102
-📄 Attached to this email, you will find your digitally signed loan agreement. We request that you review the document carefully to ensure that all details, terms, and conditions are accurate and aligned with the Sanction Letter.
-✅ If everything is in order, no further action is required. Your loan will be processed strictly in accordance with the terms outlined in the agreement.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal Initiation</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>After the loan is approved and the LAMF account is created – the customer can now initiate a withdrawal</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is XXXXXXXX.
-You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are pleased to inform you that your loan application with Shriram Credit Company Limited (SCCL) has been successfully approved, and your Loan ID is SCCLMF20261000102.
-You can now initiate the withdrawal request for the approved amount at https://lamf.shriramcredit.in/.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal Initiation: Successful LAMF Account Creation – &lt;&lt; Full Name of the customer &gt;&gt;</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Loan Disbursal Confirmation (First Disbursement)</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>When the first disbursement is credited to the customer’s bank account</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
-Loan Details:
-• Customer ID: [XXXX]
-• Loan Account ID: [XXXX]
-• Disbursement Type: &lt;&lt;Single / Multiple&gt;&gt;
-• Disbursement No.: &lt;&lt;1&gt;&gt;
-• Disbursement UTRN: [XXXX]
-• Loan Tenure: [XX months]
-• EMI Amount: ₹[XXXX]
-• First EMI Due Date: [Date]
-• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
-Repayment Schedule – 12 rows, one per month of the 12-month tenure; a 13th row is shown only when required
-Repayment Date | Repayment Amount
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-(13th row only when required) DD-MMM-YYYY | ₹XXXXXX
-Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are happy to inform you that your loan amount of ₹10,000 has been credited to your bank account.
-Loan Details:
-• Customer ID: SCCL1000102
-• Loan Account ID: SCCLMF20261000102
-• Disbursement Type: Multiple
-• Disbursement No.: 1
-• Disbursement UTRN: UTIBR52026102700001
-• Loan Tenure: 12 months
-• EMI Amount: ₹88
-• First EMI Due Date: 05-11-2026
-• Balance amount available ₹1,55,26,100 (If disbursement type is MULTIPLE.)
-Repayment Schedule – 12 rows, one per month of the 12-month tenure; a 13th row is shown only when required
-Repayment Date | Repayment Amount
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-(13th row only when required) DD-MMM-YYYY | ₹XXXXXX
-Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Loan disbursed to your account</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Loan Disbursal Confirmation (Subsequent Disbursement)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>When each later disbursement (disbursement type Multiple) is credited</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are happy to inform you that your loan amount of ₹[XXXX] has been credited to your bank account.
-Loan Details:
-• Customer ID: [XXXX]
-• Loan Account ID: [XXXX]
-• Disbursement Type: &lt;&lt;Multiple&gt;&gt;
-• Disbursement No.: 
-• Disbursement UTRN: [XXXX]
-• Loan Tenure: [XX months]
-• EMI Amount of this disbursement for 30-day cycle: ₹[XXXX]
-• First EMI Due Date: [Date]
-• Balance amount available &lt;&lt;₹&gt;&gt; (If disbursement type is MULTIPLE.)
-Repayment Schedule (display only the residual term) – cumulative of all disbursements till date
-Repayment Date | Repayment Amount
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-Please note that the purpose of the loan, as confirmed by you, is &lt;&lt;Purpose&gt;&gt; and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are happy to inform you that your loan amount of ₹20,000 has been credited to your bank account.
-Loan Details:
-• Customer ID: SCCL1000102
-• Loan Account ID: SCCLMF20261000102
-• Disbursement Type: Multiple
-• Disbursement No.: 2
-• Disbursement UTRN: UTIBR52026110200002
-• Loan Tenure: 12 months
-• EMI Amount of this disbursement for 30-day cycle: ₹175
-• First EMI Due Date: 05-12-2026
-• Balance amount available ₹1,55,06,100 (If disbursement type is MULTIPLE.)
-Repayment Schedule (display only the residual term) – cumulative of all disbursements till date
-Repayment Date | Repayment Amount
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-DD-MMM-YYYY | ₹XXXXXX
-Please note that the purpose of the loan, as confirmed by you, is Home Renovation and not for any speculative trading in securities, derivatives, commodities, or any unlawful purposes.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Loan disbursed to your account</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Upcoming EMI Due Reminder</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Sent 5 days before the original presentation of the EMI (routine T-5)</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
-Here are the details of your loan:
-• Borrowed amount: ₹ 55,000
-• Outstanding amount: ₹ 55,000
-• Bank account number: XXXXXXXXXXX
-Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
-Thank you for your cooperation.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
-Here are the details of your loan:
-• Borrowed amount: ₹ 55,000
-• Outstanding amount: ₹ 55,000
-• Bank account number: XXXXXXXXXXX
-Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
-Thank you for your cooperation.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Reminder: Your EMI of ₹[XXXX] is due on [Date]</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>EMI Presentation Mail</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Sent one day before the EMI presentation date (routine T-1)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
-Here are the details of your loan:
-• Borrowed amount: ₹ 55,000
-• Outstanding amount: ₹ 55,000
-• Bank account number: XXXXXXXXXXX
-Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
-Thank you for your cooperation.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-This is a reminder that your next EMI of Rs. 5,085 for your loan will be automatically deducted from your bank account on 10/07/2026. Kindly ensure that your account has sufficient funds to cover the payment.
-Here are the details of your loan:
-• Borrowed amount: ₹ 55,000
-• Outstanding amount: ₹ 55,000
-• Bank account number: XXXXXXXXXXX
-Please note that failure or bounce of the EMI payment may attract penal charges. We encourage you to make sure that your account balance is adequate to avoid any inconvenience.
-Thank you for your cooperation.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>EMI Presentation Alert – &lt;&lt;Date of EMI&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Successful EMI Deduction Mail</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Routine EMI clearance – the EMI is debited successfully</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are writing to confirm that your EMI of ₹[XXXX] for the loan account [Loan ID] was successfully debited on [Date] from your registered bank account.
-📄 EMI Details:
-• Loan Account Number: [Loan ID]
-• EMI Amount: ₹[XXXX]
-• Deduction Date: [Date]
-• Next EMI Due Date: [Next Date]
-Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are writing to confirm that your EMI of ₹10,000 for the loan account SCCLMF20261000102 was successfully debited on 05-11-2026 from your registered bank account.
-📄 EMI Details:
-• Loan Account Number: SCCLMF20261000102
-• EMI Amount: ₹10,000
-• Deduction Date: 05-11-2026
-• Next EMI Due Date: 05-12-2026
-Thank you for ensuring timely payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>Your EMI of ₹[XXXX] Has Been Successfully Deducted</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Instalment Failure / EMI Bounce Notification (Bounce – 1A)</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>When the EMI bounces (insufficient balance); re-presented on T+5 days</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We could not process your EMI of ₹[XXXX] for the loan account [Loan ID] on [Date] due to insufficient balance.
-We will re-present the EMI on &lt;&lt;T+5 days&gt;&gt;. Please ensure your account has a sufficient balance to avoid penalties.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We could not process your EMI of ₹10,000 for the loan account SCCLMF20261000102 on 05-11-2026 due to insufficient balance.
-We will re-present the EMI on 10-11-2026. Please ensure your account has a sufficient balance to avoid penalties.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Alert: Your EMI payment failed</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Second EMI Representation Reminder (1B T-1)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Sent one day before the EMI is re-presented</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-This is to inform you that your EMI of ₹[XXXX] will be re-presented on [Date].
-Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-This is to inform you that your EMI of ₹10,000 will be re-presented on 10-11-2026.
-Please ensure your account has a sufficient balance to avoid penalties and negative impact on your credit score.
-In case the amount is not received on the re-presentation date, we shall initiate loan closure procedures.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Final Reminder: EMI Re-presentation on [Date]</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Initiation of Loan Closure Procedures (2B Bounce)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>When the re-presented EMI bounces again – pledge liquidation is initiated</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Since you defaulted on your repayment, we are initiating the pledge liquidation process to recover the total outstanding amount.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Urgent: Mutual Fund Liquidation Scheduled</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Part Payment</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>When a part payment is processed successfully; the revised repayment schedule is attached</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
-Payment Summary:
-• Transaction Status: Successful
-• Amount Received: [₹XXXX Mention Amount]
-• Revised Outstanding Balance: [₹XXXX Mention Amount]
-Updated Repayment Schedule:
-As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We confirm that part payment towards your Loan Against Mutual Fund (LAMF) from Shriram Credit has been successfully processed.
-Payment Summary:
-• Transaction Status: Successful
-• Amount Received: ₹5,000
-• Revised Outstanding Balance: ₹5,000
-Updated Repayment Schedule:
-As a result of this payment, your Repayment Schedule has been revised. Please find the updated schedule attached to this email for your reference.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Payment Acknowledgment: Your Shriram Credit Loan Against Mutual Funds Part Payment Has Been Processed</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Pre Closure</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>When the customer pre-closes the loan (final payment received before the end of the tenure)</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Congratulations on successfully pre-closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Loan Pre-Closure Confirmation: Your Shriram Credit Loan Against Mutual Funds Has Been Closed Successfully</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Margin Call / Mutual Fund Value Drop Mail</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>When the market value of the pledged units drops and the LTV is above the limit</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-The current market value of your Mutual Fund units pledged with us has declined and current LTV is at (YY.YY)%
-We request you to make an immediate payment of ₹ (XXXX) (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of (XXXX/0.65) or For Debt MF of (XXXX/0.75)) to bring your account within the prescribed limit.
-Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
-Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
-Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your prompt attention to this matter.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-The current market value of your Mutual Fund units pledged with us has declined and current LTV is at 82.50%
-We request you to make an immediate payment of ₹ 10,000 (minimum amount) to reduce your total loan outstanding, or increase your collateral pledge (For Equity MF of ₹15,385 or For Debt MF of ₹13,333) to bring your account within the prescribed limit.
-Please visit our website and follow the easy steps to make the payment or increase your collateral pledge.
-Failure to maintain the required margin may result in loan adjustment actions as per the terms of Loan Agreement.
-Should you have any questions, require clarification, or need assistance, please feel free to reach out to our customer support team at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your prompt attention to this matter.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Mutual Fund Margin Shortfall</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Loan Tenure Completion (Closure Mail)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>EMI loan: when the last EMI is paid; balloon loan: when the principal outstanding is paid</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Congratulations on successfully closing your Loan Against Mutual Fund (LAMF) with Shriram Credit.
-We have received the final payment and are pleased to confirm that your loan account has been closed in our records. We appreciate your commitment to timely repayment and hope this facility served your financial needs effectively.
-Lien Removal Process:
-As your loan is now fully repaid, we have initiated the process to release the lien on your pledged Mutual Fund units.
-• Timeline: The lien will be removed within 2 to 3 working days.
-• Confirmation: You will receive a separate notification from the Registrar and Transfer Agent (CAMS/KFintech) once your units are fully "unlocked" and fully accessible to you.
-Next Steps:
-No Objection Certificate (NOC): Your formal No Objection Certificate is being generated and will be sent to you in a separate communication shortly.
-Important Information:
-• Please retain this email for your records as confirmation of loan closure until you receive your formal No Objection Certificate.
-• In case the lien is not removed within the stated timeline, please contact us for assistance.
-Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Congratulations on completing your loan journey</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>NOC / Loan Closure Certificate</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Manual trigger after the loan is closed; the NOC is attached</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-We are pleased to inform you that your loan account [Loan ID] has been closed successfully.
-The No Objection Certificate (NOC) is attached for your records.
-Your Customer ID is active with us, and you may visit us for any future requirements.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-We are pleased to inform you that your loan account SCCLMF20261000102 has been closed successfully.
-The No Objection Certificate (NOC) is attached for your records.
-Your Customer ID is active with us, and you may visit us for any future requirements.
-We thank you for choosing Shriram Credit and look forward to serving you again.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Your Loan Account [Loan ID] is closed successfully</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>LTV Breach beyond Policy Norms</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>When the LTV keeps breaching after the margin call and reaches the liquidation threshold</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
-Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Despite our previous communications, the Loan-to-Value (LTV) ratio of your Loan Against Mutual Funds has continued to breach the permissible limit and has now reached the liquidation threshold.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the margin shortfall, in accordance with the terms and conditions of your Loan Agreement.
-Any surplus amount, after adjustment of all outstanding dues and applicable charges, shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Principal Repayment for Loan Closure</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>When the loan reaches maturity and the outstanding principal is unpaid – 5 working days grace period</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
-As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
-Please note that:
-• Interest at the applicable contractual rate shall continue to accrue during the grace period.
-• The outstanding amount must be repaid within the stipulated grace period.
-Please use the below link to check the details and make payment.
-{LINK}
-Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
-Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
-Thank you for your prompt attention.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-Your Loan Against Mutual Funds has reached its maturity date and the outstanding principal amount remains unpaid.
-As a goodwill measure, Shriram Credit is providing a grace period of five (5) working days from the maturity date to enable you to repay the outstanding principal.
-Please note that:
-• Interest at the applicable contractual rate shall continue to accrue during the grace period.
-• The outstanding amount must be repaid within the stipulated grace period.
-Please use the below link to check the details and make payment.
-https://lamf.shriramcredit.in/user/loans/
-Failure to repay the outstanding amount within the grace period shall result in liquidation of your pledged Mutual Fund units to recover the outstanding dues in accordance with the terms of your Loan Agreement.
-Should you require any clarification or assistance, please contact us at lassupport@shriramcredit.in.
-Thank you for your prompt attention.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Principal Repayment</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Liquidation for Outstanding Loan (after grace period)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>When the grace period for the matured loan has expired and the principal is still unpaid – liquidation is initiated. (Scenario name in the document was a pasted link – to be confirmed)</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>LMS</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>SCCL</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Dear [Customer Name],
-The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
-Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Dear AZHAGARSAMY,
-The grace period provided for repayment of your matured Loan Against Mutual Funds has expired, and the outstanding principal amount remains unpaid.
-Accordingly, Shriram Credit has initiated the liquidation of your pledged Mutual Fund units to recover the outstanding loan amount, together with applicable interest, charges and other dues, in accordance with the terms of the Loan Agreement.
-Any balance amount remaining after adjustment of all outstanding dues shall be dealt with in accordance with the Loan Agreement.
-Should you require any clarification or assistance, please feel free to contact our customer support at lassupport@shriramcredit.in.
-Thank you for your understanding.
-Warm regards,
-Team Shriram Credit
-Disclaimer:
-This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>Provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K22"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Communications: summary counts (scenarios, SMS, mail) above the table and in the Excel notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4496,33 +4496,40 @@
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
+          <t>Summary – Total scenarios: 43 · SMS: 42 (25 available · 17 to be created · 8 not required) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 21 · Mail only: 1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
+          <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
+          <t>Rows in grey (SMS Status = "Not Required") are kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+          <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>

</xml_diff>

<commit_message>
Communications: Mail Status Not Required wherever SMS Status is Not Required
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,12 +58,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00B42318"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="008A8A8A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -151,7 +145,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,8 +163,8 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -896,7 +890,11 @@
       <c r="N5" s="7" t="inlineStr"/>
       <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="7" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1063,7 +1061,11 @@
       <c r="N7" s="7" t="inlineStr"/>
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="9" t="inlineStr"/>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1125,7 +1127,11 @@
       <c r="N8" s="7" t="inlineStr"/>
       <c r="O8" s="7" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1187,7 +1193,11 @@
       <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="9" t="inlineStr"/>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1356,7 +1366,11 @@
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr"/>
-      <c r="Q11" s="9" t="inlineStr"/>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1418,7 +1432,11 @@
       <c r="N12" s="7" t="inlineStr"/>
       <c r="O12" s="7" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr"/>
-      <c r="Q12" s="9" t="inlineStr"/>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1480,7 +1498,11 @@
       <c r="N13" s="7" t="inlineStr"/>
       <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="9" t="inlineStr"/>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1604,7 +1626,11 @@
       <c r="N15" s="7" t="inlineStr"/>
       <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="9" t="inlineStr"/>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
       <c r="R15" s="7" t="inlineStr"/>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Communications: SMS Status and Mail Status columns removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not Required" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS and Mail'!$A$1:$R$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not Required'!$A$1:$R$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS and Mail'!$A$1:$P$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not Required'!$A$1:$P$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,18 +42,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0012753B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00B42318"/>
       <sz val="11"/>
     </font>
@@ -66,13 +54,8 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="008A8A8A"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -87,11 +70,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -132,41 +110,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -545,14 +499,12 @@
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
     <col width="70" customWidth="1" min="14" max="14"/>
-    <col width="70" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -608,40 +560,30 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>SMS Status</t>
+          <t>Mail Subject Structure</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mail Subject Structure</t>
+          <t>Actual Mail Subject</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Actual Mail Subject</t>
+          <t>Mail Content Structure</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Mail Content Structure</t>
+          <t>Actual Mail Content</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Actual Mail Content</t>
+          <t>Mail Available</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Mail Available</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Mail Status</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -691,23 +633,17 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -753,23 +689,17 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -815,23 +745,17 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -877,27 +801,22 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
+          <t>123456 – Your Email Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>123456 – Your Email Verification OTP for Shriram Credit LAMF</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>E-Mail Verification
 Dear {{CUSTOMER_NAME}},
@@ -911,7 +830,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>E-Mail Verification
 Dear AZHAGARSAMY,
@@ -925,18 +844,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -982,14 +896,14 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Your mutual fund pledge is successful</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -998,11 +912,6 @@
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>Your mutual fund pledge is successful</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Mutual Fund Pledge Successful
 Dear {{CUSTOMER_NAME}},
@@ -1015,7 +924,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Mutual Fund Pledge Successful
 Dear AZHAGARSAMY,
@@ -1028,270 +937,241 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Both the SMS and Email communication are currently received once the loan lodgement is successful, but they are supposed to come right after the pledging is successful.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Application Expired – Lien Marked</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>The application reaches Day 31 without submission and the lien is still marked</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr"/>
-      <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="10" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
+      <c r="N7" s="5" t="inlineStr"/>
+      <c r="O7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Lien Removal Initiated</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr"/>
-      <c r="M8" s="7" t="inlineStr"/>
-      <c r="N8" s="7" t="inlineStr"/>
-      <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="10" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Lien Removal Successful</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>The lien removal confirmation is received from the RTA</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="10" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
+      <c r="N9" s="5" t="inlineStr"/>
+      <c r="O9" s="5" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Lien Removal Failed</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>The lien removal request fails or is rejected by the service provider</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr"/>
-      <c r="M10" s="7" t="inlineStr"/>
-      <c r="N10" s="7" t="inlineStr"/>
-      <c r="O10" s="7" t="inlineStr"/>
-      <c r="P10" s="7" t="inlineStr"/>
-      <c r="Q10" s="10" t="inlineStr"/>
-      <c r="R10" s="7" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" s="5" t="inlineStr"/>
+      <c r="P10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1337,27 +1217,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+          <t>SCCL Loan Sanction Letter – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Sanction Letter – AZHAGARSAMY SUBBURAJ</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1375,7 +1250,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1393,18 +1268,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1450,27 +1320,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
+          <t>SCCL Loan Agreement – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>SCCL Loan Agreement – AZHAGARSAMY SUBBURAJ</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1490,7 +1355,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1510,18 +1375,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1567,23 +1427,17 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr"/>
       <c r="P13" s="3" t="inlineStr"/>
-      <c r="Q13" s="5" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1629,27 +1483,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – {{CUSTOMER_FULL_NAME}}</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal Initiation: Successful LAMF Account Creation – {{CUSTOMER_FULL_NAME}}</t>
+          <t>Withdrawal Initiation: Successful LAMF Account Creation – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>Withdrawal Initiation: Successful LAMF Account Creation – AZHAGARSAMY SUBBURAJ</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>Loan Approved
 Dear {{CUSTOMER_NAME}},
@@ -1665,7 +1514,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>Loan Approved
 Dear AZHAGARSAMY,
@@ -1681,142 +1530,125 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (with payment link)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITH payment link, when the customer has charges to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="inlineStr"/>
-      <c r="N15" s="7" t="inlineStr"/>
-      <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="10" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr"/>
+      <c r="M15" s="5" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr"/>
+      <c r="O15" s="5" t="inlineStr"/>
+      <c r="P15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (without payment link)</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITHOUT payment link, when there are no charges for the customer to pay. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L16" s="7" t="inlineStr"/>
-      <c r="M16" s="7" t="inlineStr"/>
-      <c r="N16" s="7" t="inlineStr"/>
-      <c r="O16" s="7" t="inlineStr"/>
-      <c r="P16" s="7" t="inlineStr"/>
-      <c r="Q16" s="10" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr"/>
+      <c r="O16" s="5" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1862,27 +1694,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>{{OTP}} – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>{{OTP}} – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
+          <t>123456 – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
-        <is>
-          <t>123456 – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
-        </is>
-      </c>
-      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>Withdrawal Verification
 Dear {{CUSTOMER_NAME}},
@@ -1896,7 +1723,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>Withdrawal Verification
 Dear AZHAGARSAMY,
@@ -1910,18 +1737,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1967,89 +1789,77 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="3" t="inlineStr"/>
-      <c r="Q18" s="5" t="inlineStr"/>
-      <c r="R18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>This SMS has to come once the withdrawal OTP is verified successfully, but it currently comes only once the UTR is approved in the LMS.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Withdrawal Rejected</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>The withdrawal status changes to Rejected after the Operations or Treasury team rejects it</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request of Rs. {#alphanumeric#} for loan account {#alphanumeric#} has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J19" s="9" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L19" s="7" t="inlineStr"/>
-      <c r="M19" s="7" t="inlineStr"/>
-      <c r="N19" s="7" t="inlineStr"/>
-      <c r="O19" s="7" t="inlineStr"/>
-      <c r="P19" s="7" t="inlineStr"/>
-      <c r="Q19" s="10" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr"/>
+      <c r="N19" s="5" t="inlineStr"/>
+      <c r="O19" s="5" t="inlineStr"/>
+      <c r="P19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2095,14 +1905,14 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Loan disbursed to your account</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -2111,11 +1921,6 @@
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>Loan disbursed to your account</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>Loan Disbursed
 Dear {{CUSTOMER_NAME}},
@@ -2153,7 +1958,7 @@
 This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>Loan Disbursed
 Dear AZHAGARSAMY,
@@ -2191,17 +1996,12 @@
 This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="P20" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q20" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>In the disbursement mail, Disbursement No. ({{DISBURSEMENT_NO}}) and Disbursement UTRN ({{UTRN}}) currently show a random format; the format of both has to be defined correctly.</t>
         </is>
@@ -2251,14 +2051,14 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Loan disbursed to your account</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -2267,11 +2067,6 @@
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Loan disbursed to your account</t>
-        </is>
-      </c>
-      <c r="N21" s="3" t="inlineStr">
         <is>
           <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
 Loan Disbursed
@@ -2301,7 +2096,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr">
+      <c r="N21" s="3" t="inlineStr">
         <is>
           <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
 Loan Disbursed
@@ -2331,18 +2126,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2388,27 +2178,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Reminder: Your EMI of ₹{{EMI_AMOUNT}} is due on {{DUE_DATE}}</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Reminder: Your EMI of ₹{{EMI_AMOUNT}} is due on {{DUE_DATE}}</t>
+          <t>Reminder: Your EMI of ₹10,000 is due on 05-11-2026</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>Reminder: Your EMI of ₹10,000 is due on 05-11-2026</t>
-        </is>
-      </c>
-      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>EMI Due Reminder
 Dear {{CUSTOMER_NAME}},
@@ -2425,7 +2210,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>EMI Due Reminder
 Dear AZHAGARSAMY,
@@ -2442,84 +2227,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>EMI Presentation Reminder (T-1)</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>This communication has to be triggered 1 day before the EMI presentation date (T-1), i.e. on the 4th when the EMI is due on the 5th – SMS and mail. SMS template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} for loan account {#alphanumeric#} will be presented tomorrow, {#alphanumeric#}. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 for loan account SCCLMF20261000102 will be presented tomorrow, 05-11-2026. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J23" s="9" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – {{DATE}}</t>
         </is>
       </c>
-      <c r="M23" s="7" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – 05-11-2026</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
+      <c r="M23" s="5" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2537,7 +2312,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2555,18 +2330,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P23" s="7" t="inlineStr">
+      <c r="O23" s="5" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="P23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2612,27 +2382,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Your EMI of ₹{{EMI_AMOUNT}} Has Been Successfully Deducted</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>Your EMI of ₹{{EMI_AMOUNT}} Has Been Successfully Deducted</t>
+          <t>Your EMI of ₹10,000 Has Been Successfully Deducted</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>Your EMI of ₹10,000 Has Been Successfully Deducted</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>EMI Payment Confirmed
 Dear {{CUSTOMER_NAME}},
@@ -2651,7 +2416,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>EMI Payment Confirmed
 Dear AZHAGARSAMY,
@@ -2670,18 +2435,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>In the mail, “Next EMI Due Date: {{NEXT_EMI_DATE}}” – what is shown for the last EMI (12th EMI), when there is no next EMI, has to be defined.</t>
         </is>
@@ -2731,27 +2491,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Alert: Your EMI payment failed {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Alert: Your EMI payment failed {{LOAN_ID}}</t>
+          <t>Alert: Your EMI payment failed SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>Alert: Your EMI payment failed SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
 Instalment Failure / EMI Bounce Notification (Bounce - 1A)
@@ -2766,7 +2521,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O25" s="3" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
 Instalment Failure / EMI Bounce Notification (Bounce - 1A)
@@ -2781,18 +2536,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="O25" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q25" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R25" s="3" t="inlineStr">
+      <c r="P25" s="3" t="inlineStr">
         <is>
           <t>In the mail, the title “Instalment Failure / EMI Bounce Notification (Bounce - 1A)” has to be changed to “EMI Payment Failed”.</t>
         </is>
@@ -2842,27 +2592,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Final Reminder: EMI Re-presentation on {{REPRESENTATION_DATE}} &lt;&lt;{{LOAN_ID}}&gt;&gt;</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Final Reminder: EMI Re-presentation on {{REPRESENTATION_DATE}} &lt;&lt;{{LOAN_ID}}&gt;&gt;</t>
+          <t>Final Reminder: EMI Re-presentation on 10-11-2026 SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Final Reminder: EMI Re-presentation on 10-11-2026 SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
 Second EMI Representation Reminder (1B T-1)
@@ -2876,7 +2621,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
 Second EMI Representation Reminder (1B T-1)
@@ -2890,18 +2635,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2947,23 +2687,17 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="K27" s="3" t="inlineStr"/>
       <c r="L27" s="3" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr"/>
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr"/>
       <c r="P27" s="3" t="inlineStr"/>
-      <c r="Q27" s="5" t="inlineStr"/>
-      <c r="R27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -3009,27 +2743,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Urgent: Mutual Fund Liquidation Scheduled {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>Urgent: Mutual Fund Liquidation Scheduled {{LOAN_ID}}</t>
+          <t>Urgent: Mutual Fund Liquidation Scheduled SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Urgent: Mutual Fund Liquidation Scheduled SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>Initiation of Loan Closure Procedures (2B Bounce)
 Dear {{CUSTOMER_NAME}},
@@ -3041,7 +2770,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>Initiation of Loan Closure Procedures (2B Bounce)
 Dear AZHAGARSAMY,
@@ -3053,18 +2782,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -3110,14 +2834,14 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -3126,11 +2850,6 @@
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
-        </is>
-      </c>
-      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>Attachment: Updated Repayment Schedule PDF
 Part Payment Processed
@@ -3149,7 +2868,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>Attachment: Updated Repayment Schedule PDF
 Part Payment Processed
@@ -3168,18 +2887,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -3225,27 +2939,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Action Required: Mutual Fund Margin Shortfall &lt;&lt;Loan ID&gt;&gt;</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Action Required: Mutual Fund Margin Shortfall &lt;&lt;Loan ID&gt;&gt;</t>
+          <t>Action Required: Mutual Fund Margin Shortfall SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Mutual Fund Margin Shortfall SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>Trigger: LTV breach – notifying the customer of a margin shortfall
 Margin Call / Mutual Fund Value Drop
@@ -3262,7 +2971,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>Trigger: LTV breach – notifying the customer of a margin shortfall
 Margin Call / Mutual Fund Value Drop
@@ -3279,18 +2988,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -3336,27 +3040,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach {{LOAN_ID}}</t>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>LTV Breach – Liquidation of Pledged Units
 Dear {{CUSTOMER_NAME}},
@@ -3371,7 +3070,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>LTV Breach – Liquidation of Pledged Units
 Dear AZHAGARSAMY,
@@ -3386,18 +3085,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3443,27 +3137,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Action Required: Principal Repayment {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>Action Required: Principal Repayment {{LOAN_ID}}</t>
+          <t>Action Required: Principal Repayment SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Action Required: Principal Repayment SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>Principal Repayment for Loan Closure
 Dear {{CUSTOMER_NAME}},
@@ -3483,7 +3172,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>Principal Repayment for Loan Closure
 Dear AZHAGARSAMY,
@@ -3503,18 +3192,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3560,27 +3244,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan {{LOAN_ID}}</t>
+          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan SCCLMF20261000102</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
         <is>
           <t>Liquidation for Outstanding Loan
 Dear {{CUSTOMER_NAME}},
@@ -3595,7 +3274,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O33" s="3" t="inlineStr">
+      <c r="N33" s="3" t="inlineStr">
         <is>
           <t>Liquidation for Outstanding Loan
 Dear AZHAGARSAMY,
@@ -3610,84 +3289,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P33" s="3" t="inlineStr">
+      <c r="O33" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R33" s="3" t="inlineStr"/>
+      <c r="P33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Foreclosure Completed</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I34" s="8" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J34" s="9" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="L34" s="7" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
         </is>
       </c>
-      <c r="M34" s="7" t="inlineStr">
+      <c r="L34" s="5" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
         </is>
       </c>
-      <c r="N34" s="7" t="inlineStr">
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation
 Dear {{CUSTOMER_NAME}},
@@ -3711,7 +3380,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O34" s="7" t="inlineStr">
+      <c r="N34" s="5" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation
 Dear AZHAGARSAMY,
@@ -3735,18 +3404,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P34" s="7" t="inlineStr">
+      <c r="O34" s="5" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q34" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R34" s="7" t="inlineStr"/>
+      <c r="P34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3792,14 +3456,14 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Congratulations on completing your loan journey</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
@@ -3808,11 +3472,6 @@
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Congratulations on completing your loan journey</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
         <is>
           <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
 Loan Journey Complete
@@ -3837,7 +3496,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr">
+      <c r="N35" s="3" t="inlineStr">
         <is>
           <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
 Loan Journey Complete
@@ -3862,18 +3521,13 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P35" s="3" t="inlineStr">
+      <c r="O35" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q35" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R35" s="3" t="inlineStr"/>
+      <c r="P35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3919,27 +3573,22 @@
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Your Loan Account {{LOAN_ID}} is closed successfully</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>Your Loan Account {{LOAN_ID}} is closed successfully</t>
+          <t>Your Loan Account SCCLMF20261000102 is closed successfully</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Your Loan Account SCCLMF20261000102 is closed successfully</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr">
         <is>
           <t>Trigger: manual trigger
 Attachment: NOC / Loan Closure Certificate PDF
@@ -3956,7 +3605,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr">
+      <c r="N36" s="3" t="inlineStr">
         <is>
           <t>Trigger: manual trigger
 Attachment: NOC / Loan Closure Certificate PDF
@@ -3973,92 +3622,87 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="P36" s="3" t="inlineStr">
+      <c r="O36" s="3" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="Q36" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="R36" s="3" t="inlineStr"/>
+      <c r="P36" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t>Rows with SMS Status = "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>SMS and mail marked "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R36"/>
+  <autoFilter ref="A1:P36"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4071,7 +3715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4084,14 +3728,12 @@
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
     <col width="70" customWidth="1" min="14" max="14"/>
-    <col width="70" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4147,624 +3789,534 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>SMS Status</t>
+          <t>Mail Subject Structure</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mail Subject Structure</t>
+          <t>Actual Mail Subject</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Actual Mail Subject</t>
+          <t>Mail Content Structure</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Mail Content Structure</t>
+          <t>Actual Mail Content</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Actual Mail Content</t>
+          <t>Mail Available</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Mail Available</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Mail Status</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>LAN Generated</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>When the customer clicks Continue on the Loan Application Summary page and the Loan Account Number (LAN) is generated successfully</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is {#alphanumeric#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L2" s="14" t="inlineStr"/>
-      <c r="M2" s="14" t="inlineStr"/>
-      <c r="N2" s="14" t="inlineStr"/>
-      <c r="O2" s="14" t="inlineStr"/>
-      <c r="P2" s="14" t="inlineStr"/>
-      <c r="Q2" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R2" s="14" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K3" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L3" s="14" t="inlineStr"/>
-      <c r="M3" s="14" t="inlineStr"/>
-      <c r="N3" s="14" t="inlineStr"/>
-      <c r="O3" s="14" t="inlineStr"/>
-      <c r="P3" s="14" t="inlineStr"/>
-      <c r="Q3" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R3" s="14" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
+      <c r="N3" s="5" t="inlineStr"/>
+      <c r="O3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Discarded</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr"/>
-      <c r="M4" s="14" t="inlineStr"/>
-      <c r="N4" s="14" t="inlineStr"/>
-      <c r="O4" s="14" t="inlineStr"/>
-      <c r="P4" s="14" t="inlineStr"/>
-      <c r="Q4" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R4" s="14" t="inlineStr"/>
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr"/>
+      <c r="O4" s="5" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Customer-Initiated Discard</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr"/>
-      <c r="M5" s="14" t="inlineStr"/>
-      <c r="N5" s="14" t="inlineStr"/>
-      <c r="O5" s="14" t="inlineStr"/>
-      <c r="P5" s="14" t="inlineStr"/>
-      <c r="Q5" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R5" s="14" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="inlineStr"/>
+      <c r="O5" s="5" t="inlineStr"/>
+      <c r="P5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Lien Marking Failed</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J6" s="15" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="inlineStr"/>
-      <c r="M6" s="14" t="inlineStr"/>
-      <c r="N6" s="14" t="inlineStr"/>
-      <c r="O6" s="14" t="inlineStr"/>
-      <c r="P6" s="14" t="inlineStr"/>
-      <c r="Q6" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R6" s="14" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Post-Pledge Journey Incomplete</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Lien marking is successful, then the customer is inactive for the configured period</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J7" s="15" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L7" s="14" t="inlineStr"/>
-      <c r="M7" s="14" t="inlineStr"/>
-      <c r="N7" s="14" t="inlineStr"/>
-      <c r="O7" s="14" t="inlineStr"/>
-      <c r="P7" s="14" t="inlineStr"/>
-      <c r="Q7" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R7" s="14" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
+      <c r="N7" s="5" t="inlineStr"/>
+      <c r="O7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Post-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="15" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr"/>
-      <c r="M8" s="14" t="inlineStr"/>
-      <c r="N8" s="14" t="inlineStr"/>
-      <c r="O8" s="14" t="inlineStr"/>
-      <c r="P8" s="14" t="inlineStr"/>
-      <c r="Q8" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R8" s="14" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Lien Removal Request Received</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>SCCL receives and records the customer’s lien removal request</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="15" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="L9" s="14" t="inlineStr"/>
-      <c r="M9" s="14" t="inlineStr"/>
-      <c r="N9" s="14" t="inlineStr"/>
-      <c r="O9" s="14" t="inlineStr"/>
-      <c r="P9" s="14" t="inlineStr"/>
-      <c r="Q9" s="16" t="inlineStr">
-        <is>
-          <t>Not Required</t>
-        </is>
-      </c>
-      <c r="R9" s="14" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
+      <c r="N9" s="5" t="inlineStr"/>
+      <c r="O9" s="5" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Rows with SMS Status = "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>SMS and mail marked "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R9"/>
+  <autoFilter ref="A1:P9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Communications: General / SMS / Mail column group header row (page and Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not Required" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS and Mail'!$A$1:$P$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not Required'!$A$1:$P$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SMS and Mail'!$A$2:$P$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not Required'!$A$2:$P$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,13 +21,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -55,7 +60,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +70,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B4C6E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,28 +129,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -510,313 +558,347 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="n"/>
+      <c r="M1" s="6" t="n"/>
+      <c r="N1" s="6" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Scenarios</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Sender</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Communication Type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>SMS Content Structure</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Actual SMS Content</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>SMS Header</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>SMS Available</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Mail Subject Structure</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Actual Mail Subject</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Mail Content Structure</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>Actual Mail Content</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>Mail Available</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="3">
+      <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Enter Mobile Number Page</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>After entered the mobile number and user clicking the “Continue” CTA on “Enter your MF linked Mobile Number” page</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>{#numeric#} is your OTP to sign in to Shriram Credit Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>123456 is your OTP to sign in to Shriram Credit Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="K3" s="11" t="inlineStr"/>
+      <c r="L3" s="11" t="inlineStr"/>
+      <c r="M3" s="11" t="inlineStr"/>
+      <c r="N3" s="11" t="inlineStr"/>
+      <c r="O3" s="11" t="inlineStr"/>
+      <c r="P3" s="11" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Mutual Fund Portfolio fetching in MF Central</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>After clicked the “Check Credit Limit” CTA in “LOS to MF Central Redirection consent page” then in MF central, there is no data available the combination of “mobile number” and “PAN Number”</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, No Mutual Fund investments were found for the details you provided. Please verify your credentials and try again - Shriram Credit</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, No Mutual Fund investments were found for the details you provided. Please verify your credentials and try again - Shriram Credit</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="K4" s="11" t="inlineStr"/>
+      <c r="L4" s="11" t="inlineStr"/>
+      <c r="M4" s="11" t="inlineStr"/>
+      <c r="N4" s="11" t="inlineStr"/>
+      <c r="O4" s="11" t="inlineStr"/>
+      <c r="P4" s="11" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Applying SCCL’s Eligibility Business Rule Engine (BRE)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>After fetched mutual fund portfolio from MF central then applying SCCL’s eligibility BRE, as per BRE users not eligible</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your loan request could not be approved per our policy. For assistance, contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your loan request could not be approved per our policy. For assistance, contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="K5" s="11" t="inlineStr"/>
+      <c r="L5" s="11" t="inlineStr"/>
+      <c r="M5" s="11" t="inlineStr"/>
+      <c r="N5" s="11" t="inlineStr"/>
+      <c r="O5" s="11" t="inlineStr"/>
+      <c r="P5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Email Verification</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>On the KYC Verification page (LOS step 9, after the Application Summary): the customer enters the email address and clicks Verify, and the OTP is sent to that email</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Mail</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>XXXXXX – Your Email Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>123456 – Your Email Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>E-Mail Verification
 Dear {{CUSTOMER_NAME}},
@@ -830,7 +912,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>E-Mail Verification
 Dear AZHAGARSAMY,
@@ -844,74 +926,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O6" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="P6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Pledging of Mutual Fund</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>After the mutual fund units are successfully pledged on the “Pledging of Mutual Fund” page (Pledge Securities → MF Central OTP → “Successfully pledged!”)</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Mutual Fund units have been successfully pledged against your loan with Shriram Credit. You may now proceed further - Shriram Credit</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Your mutual fund pledge is successful</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>Your mutual fund pledge is successful</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M7" s="11" t="inlineStr">
         <is>
           <t>Mutual Fund Pledge Successful
 Dear {{CUSTOMER_NAME}},
@@ -924,7 +1006,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>Mutual Fund Pledge Successful
 Dear AZHAGARSAMY,
@@ -937,302 +1019,302 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O7" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="P7" s="11" t="inlineStr">
         <is>
           <t>Both the SMS and Email communication are currently received once the loan lodgement is successful, but they are supposed to come right after the pledging is successful.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+    <row r="8">
+      <c r="A8" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Application Expired – Lien Marked</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>The application reaches Day 31 without submission and the lien is still marked</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
-      <c r="O7" s="5" t="inlineStr"/>
-      <c r="P7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="K8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="13" t="inlineStr"/>
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Lien Removal Initiated</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>SCCL initiates the lien removal through the applicable RTA / MF Central process</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal has been initiated for the Mutual Fund units pledged against loan account {#alphanumeric#}. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="K9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="13" t="inlineStr"/>
+      <c r="O9" s="13" t="inlineStr"/>
+      <c r="P9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Lien Removal Successful</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>The lien removal confirmation is received from the RTA</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, The lien on your Mutual Fund units pledged against loan account {#alphanumeric#} has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr"/>
-      <c r="O9" s="5" t="inlineStr"/>
-      <c r="P9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="K10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="13" t="inlineStr"/>
+      <c r="P10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Lien Removal Failed</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>The lien removal request fails or is rejected by the service provider</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien removal for loan account {#alphanumeric#} could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr"/>
-      <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="K11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="13" t="inlineStr"/>
+      <c r="N11" s="13" t="inlineStr"/>
+      <c r="O11" s="13" t="inlineStr"/>
+      <c r="P11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Sanction Letter</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>After the Sanction Letter is generated successfully (customer clicks “Sign Agreement” on the “Agreement and E-Mandate” page and the Sanction Letter is generated)</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund has been sanctioned. Your Sanction Letter will be shared separately. Please proceed to sign the eAgreement to continue your loan journey - Shriram Credit</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>SCCL Loan Sanction Letter – &lt;&lt; Full Name of the customer &gt;&gt;</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>SCCL Loan Sanction Letter – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M12" s="11" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1250,7 +1332,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1268,74 +1350,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O12" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="P12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Loan Agreement e-Sign</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>After the customer signs the loan agreement successfully (e-Sign at Digio – Aadhaar / VID + OTP → “Signed Successfully”)</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully processed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>SCCL Loan Agreement – &lt;&lt; Full Name of the customer &gt;&gt;</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>SCCL Loan Agreement – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M13" s="11" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1355,7 +1437,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>To: Customer Email ID
 CC: loandocuments@shriramcredit.in
@@ -1375,130 +1457,130 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O13" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="P13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>LAMF Application Submit</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr"/>
-      <c r="O13" s="3" t="inlineStr"/>
-      <c r="P13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="K14" s="11" t="inlineStr"/>
+      <c r="L14" s="11" t="inlineStr"/>
+      <c r="M14" s="11" t="inlineStr"/>
+      <c r="N14" s="11" t="inlineStr"/>
+      <c r="O14" s="11" t="inlineStr"/>
+      <c r="P14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Loan Lodgement Approval</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>After the application is submitted, the OPS team approves in the backend LMS, back to back: first the Loan Account Opening approval, then the Loan Lodgement approval. This SMS is triggered when the Loan Lodgement is approved</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Shriram Credit - Loan Against Mutual Fund is approved and active. Withdraw your funds now:- https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>Withdrawal Initiation: Successful LAMF Account Creation – {{CUSTOMER_FULL_NAME}}</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>Withdrawal Initiation: Successful LAMF Account Creation – AZHAGARSAMY SUBBURAJ</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>Loan Approved
 Dear {{CUSTOMER_NAME}},
@@ -1514,7 +1596,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>Loan Approved
 Dear AZHAGARSAMY,
@@ -1530,186 +1612,186 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="O15" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="P15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (with payment link)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITH payment link, when the customer has charges to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. {#alphanumeric#} using this link: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr"/>
-      <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr"/>
-      <c r="O15" s="5" t="inlineStr"/>
-      <c r="P15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="K16" s="13" t="inlineStr"/>
+      <c r="L16" s="13" t="inlineStr"/>
+      <c r="M16" s="13" t="inlineStr"/>
+      <c r="N16" s="13" t="inlineStr"/>
+      <c r="O16" s="13" t="inlineStr"/>
+      <c r="P16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Loan Account Opening / Loan Lodgement Rejection (without payment link)</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITHOUT payment link, when there are no charges for the customer to pay. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr"/>
-      <c r="M16" s="5" t="inlineStr"/>
-      <c r="N16" s="5" t="inlineStr"/>
-      <c r="O16" s="5" t="inlineStr"/>
-      <c r="P16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="K17" s="13" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr"/>
+      <c r="M17" s="13" t="inlineStr"/>
+      <c r="N17" s="13" t="inlineStr"/>
+      <c r="O17" s="13" t="inlineStr"/>
+      <c r="P17" s="13" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>When the customer initiates a withdrawal from the loan account, an OTP is sent to confirm the withdrawal</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>{#numeric#} is your OTP to confirm the withdrawal of Rs. {#alphanumeric#} from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>123456 is your OTP to confirm the withdrawal of Rs. 10,000 from your Loan Against Mutual Fund. Do not share this OTP with anyone - Shriram Credit</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J18" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>{{OTP}} – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="L18" s="11" t="inlineStr">
         <is>
           <t>123456 – Your Withdrawal Verification OTP for Shriram Credit LAMF</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M18" s="11" t="inlineStr">
         <is>
           <t>Withdrawal Verification
 Dear {{CUSTOMER_NAME}},
@@ -1723,7 +1805,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="N18" s="11" t="inlineStr">
         <is>
           <t>Withdrawal Verification
 Dear AZHAGARSAMY,
@@ -1737,190 +1819,190 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="O18" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="P18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-      <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr"/>
+      <c r="L19" s="11" t="inlineStr"/>
+      <c r="M19" s="11" t="inlineStr"/>
+      <c r="N19" s="11" t="inlineStr"/>
+      <c r="O19" s="11" t="inlineStr"/>
+      <c r="P19" s="11" t="inlineStr">
         <is>
           <t>This SMS has to come once the withdrawal OTP is verified successfully, but it currently comes only once the UTR is approved in the LMS.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
+    <row r="20">
+      <c r="A20" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Withdrawal Rejected</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>The withdrawal status changes to Rejected after the Operations or Treasury team rejects it</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request of Rs. {#alphanumeric#} for loan account {#alphanumeric#} has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H20" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I20" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J20" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr"/>
-      <c r="M19" s="5" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr"/>
-      <c r="O19" s="5" t="inlineStr"/>
-      <c r="P19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="K20" s="13" t="inlineStr"/>
+      <c r="L20" s="13" t="inlineStr"/>
+      <c r="M20" s="13" t="inlineStr"/>
+      <c r="N20" s="13" t="inlineStr"/>
+      <c r="O20" s="13" t="inlineStr"/>
+      <c r="P20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Loan Disbursed (First Disbursement)</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>When the loan is disbursed for the first time (first disbursement) – notifying the customer that the amount is credited to the bank account. Each subsequent withdrawal is the row below (same SMS, different mail)</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>Loan disbursed to your account</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="L21" s="11" t="inlineStr">
         <is>
           <t>Loan disbursed to your account</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M21" s="11" t="inlineStr">
         <is>
           <t>Loan Disbursed
 Dear {{CUSTOMER_NAME}},
@@ -1958,7 +2040,7 @@
 This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="N21" s="11" t="inlineStr">
         <is>
           <t>Loan Disbursed
 Dear AZHAGARSAMY,
@@ -1996,77 +2078,77 @@
 This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="O21" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="P21" s="11" t="inlineStr">
         <is>
           <t>In the disbursement mail, Disbursement No. ({{DISBURSEMENT_NO}}) and Disbursement UTRN ({{UTRN}}) currently show a random format; the format of both has to be defined correctly.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Loan Disbursed (Subsequent Disbursement)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>On each subsequent withdrawal / disbursement after the first one – notifying the customer that the amount is credited to the bank account. Same SMS as the first disbursement (row above); only the mail is different</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Congratulations! Your loan has been credited to your bank account. Thank you for choosing Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>Loan disbursed to your account</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="L22" s="11" t="inlineStr">
         <is>
           <t>Loan disbursed to your account</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="M22" s="11" t="inlineStr">
         <is>
           <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
 Loan Disbursed
@@ -2096,7 +2178,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N21" s="3" t="inlineStr">
+      <c r="N22" s="11" t="inlineStr">
         <is>
           <t>Trigger: each subsequent disbursement (Disbursement Type: Multiple); the repayment schedule shows the residual term only
 Loan Disbursed
@@ -2126,74 +2208,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr">
+      <c r="O22" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="P22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>EMI Presentation Reminder (T-5)</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>This communication has to be triggered on the 1st of every month when the EMI is due on the 5th – first reminder of the upcoming instalment (SMS and mail). The second reminder, T-1, is mail only (next row)</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} is due on {#alphanumeric#}. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 is due on 05-11-2026. Please ensure sufficient balance in your bank account for timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>Reminder: Your EMI of ₹{{EMI_AMOUNT}} is due on {{DUE_DATE}}</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="L23" s="11" t="inlineStr">
         <is>
           <t>Reminder: Your EMI of ₹10,000 is due on 05-11-2026</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="M23" s="11" t="inlineStr">
         <is>
           <t>EMI Due Reminder
 Dear {{CUSTOMER_NAME}},
@@ -2210,7 +2292,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="N23" s="11" t="inlineStr">
         <is>
           <t>EMI Due Reminder
 Dear AZHAGARSAMY,
@@ -2227,74 +2309,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="O23" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="P23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>EMI Presentation Reminder (T-1)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>This communication has to be triggered 1 day before the EMI presentation date (T-1), i.e. on the 4th when the EMI is due on the 5th – SMS and mail. SMS template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} for loan account {#alphanumeric#} will be presented tomorrow, {#alphanumeric#}. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H24" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 for loan account SCCLMF20261000102 will be presented tomorrow, 05-11-2026. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="I24" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="J24" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K24" s="13" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – {{DATE}}</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="L24" s="13" t="inlineStr">
         <is>
           <t>EMI Presentation Alert – 05-11-2026</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M24" s="13" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2312,7 +2394,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N23" s="5" t="inlineStr">
+      <c r="N24" s="13" t="inlineStr">
         <is>
           <t>Trigger: 1 day before the EMI presentation date (T-1)
 EMI Presentation Alert
@@ -2330,74 +2412,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O23" s="5" t="inlineStr">
+      <c r="O24" s="13" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="P24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>EMI Success</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Notifying the customer when the instalment is debited successfully</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 05-11-2026. Thank you for your timely payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>Your EMI of ₹{{EMI_AMOUNT}} Has Been Successfully Deducted</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="L25" s="11" t="inlineStr">
         <is>
           <t>Your EMI of ₹10,000 Has Been Successfully Deducted</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="M25" s="11" t="inlineStr">
         <is>
           <t>EMI Payment Confirmed
 Dear {{CUSTOMER_NAME}},
@@ -2416,7 +2498,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="N25" s="11" t="inlineStr">
         <is>
           <t>EMI Payment Confirmed
 Dear AZHAGARSAMY,
@@ -2435,78 +2517,78 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="O25" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="P25" s="11" t="inlineStr">
         <is>
           <t>In the mail, “Next EMI Due Date: {{NEXT_EMI_DATE}}” – what is shown for the last EMI (12th EMI), when there is no next EMI, has to be defined.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="26">
+      <c r="A26" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>EMI Failed</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>When the EMI presentation fails on the 5th of the month, this communication has to be sent to the customer – SMS and mail</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected by your bank on {#alphanumeric#}. We will retry on {#alphanumeric#}. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected by your bank on 05-11-2026. We will retry on 10-11-2026. Please ensure sufficient balance - Shriram Credit</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>Alert: Your EMI payment failed {{LOAN_ID}}</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>Alert: Your EMI payment failed SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="M26" s="11" t="inlineStr">
         <is>
           <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
 Instalment Failure / EMI Bounce Notification (Bounce - 1A)
@@ -2521,7 +2603,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="N26" s="11" t="inlineStr">
         <is>
           <t>Trigger: EMI presented on the 5th of the month bounces (Bounce - 1A); re-presented on the 10th
 Instalment Failure / EMI Bounce Notification (Bounce - 1A)
@@ -2536,78 +2618,78 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O25" s="3" t="inlineStr">
+      <c r="O26" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="P26" s="11" t="inlineStr">
         <is>
           <t>In the mail, the title “Instalment Failure / EMI Bounce Notification (Bounce - 1A)” has to be changed to “EMI Payment Failed”.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+    <row r="27">
+      <c r="A27" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>EMI Resubmission Reminder</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>Notifying the customer before the bounced EMI is re-presented (resubmitted) to the bank – this communication has to be triggered 1 day before the re-presentation date (T-1), i.e. on the 9th when the EMI is re-presented on the 10th – SMS and mail</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} will be re-presented on {#alphanumeric#}. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 will be re-presented on 10-11-2026. Please ensure sufficient balance to avoid any disruption - Shriram Credit</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I27" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J27" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Final Reminder: EMI Re-presentation on {{REPRESENTATION_DATE}} &lt;&lt;{{LOAN_ID}}&gt;&gt;</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="L27" s="11" t="inlineStr">
         <is>
           <t>Final Reminder: EMI Re-presentation on 10-11-2026 SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="M27" s="11" t="inlineStr">
         <is>
           <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
 Second EMI Representation Reminder (1B T-1)
@@ -2621,7 +2703,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="N27" s="11" t="inlineStr">
         <is>
           <t>Trigger: 1 day prior to the EMI re-presentation (1B T-1)
 Second EMI Representation Reminder (1B T-1)
@@ -2635,130 +2717,130 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr">
+      <c r="O27" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="P27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>EMI Resubmission Success</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="J28" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
-      <c r="N27" s="3" t="inlineStr"/>
-      <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="K28" s="11" t="inlineStr"/>
+      <c r="L28" s="11" t="inlineStr"/>
+      <c r="M28" s="11" t="inlineStr"/>
+      <c r="N28" s="11" t="inlineStr"/>
+      <c r="O28" s="11" t="inlineStr"/>
+      <c r="P28" s="11" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>EMI Resubmission Failed</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Notifying the customer when the EMI resubmission fails (rejected again by the bank)</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was rejected again by your bank on {#alphanumeric#}. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was rejected again by your bank on 10-11-2026. Please check your registered email for further details - Shriram Credit</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="I29" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="J29" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>Urgent: Mutual Fund Liquidation Scheduled {{LOAN_ID}}</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="L29" s="11" t="inlineStr">
         <is>
           <t>Urgent: Mutual Fund Liquidation Scheduled SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="M29" s="11" t="inlineStr">
         <is>
           <t>Initiation of Loan Closure Procedures (2B Bounce)
 Dear {{CUSTOMER_NAME}},
@@ -2770,7 +2852,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="N29" s="11" t="inlineStr">
         <is>
           <t>Initiation of Loan Closure Procedures (2B Bounce)
 Dear AZHAGARSAMY,
@@ -2782,74 +2864,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="O29" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="P29" s="11" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>LAMF Part Payment Confirmation</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>When the customer makes a part payment towards the loan and it is processed successfully</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Part payment of Rs. {#alp#} towards your LAMF has been successfully processed. Revised outstanding: Rs. {#alp#}. - Shriram Credit</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Part payment of Rs. 5,000 towards your LAMF has been successfully processed. Revised outstanding: Rs. 5,000. - Shriram Credit</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="L30" s="11" t="inlineStr">
         <is>
           <t>Payment Acknowledgment: Your Shriram Credit LAMF Part Payment Has Been Processed</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="M30" s="11" t="inlineStr">
         <is>
           <t>Attachment: Updated Repayment Schedule PDF
 Part Payment Processed
@@ -2868,7 +2950,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="N30" s="11" t="inlineStr">
         <is>
           <t>Attachment: Updated Repayment Schedule PDF
 Part Payment Processed
@@ -2887,74 +2969,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="O30" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="P30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>LTV Breach Trigger (Margin Call)</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>When the loan-to-value (LTV) is breached because the value of the pledged portfolio has dropped – the customer is asked to pay or pledge more</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your loan value has dropped. Please pay or pledge immediately to avoid liquidation of your portfolio. https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I31" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr">
+      <c r="J31" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K31" s="11" t="inlineStr">
         <is>
           <t>Action Required: Mutual Fund Margin Shortfall &lt;&lt;Loan ID&gt;&gt;</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="L31" s="11" t="inlineStr">
         <is>
           <t>Action Required: Mutual Fund Margin Shortfall SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="M31" s="11" t="inlineStr">
         <is>
           <t>Trigger: LTV breach – notifying the customer of a margin shortfall
 Margin Call / Mutual Fund Value Drop
@@ -2971,7 +3053,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="N31" s="11" t="inlineStr">
         <is>
           <t>Trigger: LTV breach – notifying the customer of a margin shortfall
 Margin Call / Mutual Fund Value Drop
@@ -2988,74 +3070,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="O31" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="P31" s="11" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>LAMF LTV Breach Liquidation</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>When the LTV breach is not cured – liquidation of the pledged securities is initiated as per the loan terms to recover the shortfall</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your LTV has breached. As per the loan terms, liquidation of your pledged securities will be initiated to recover the shortfall - Shriram Credit</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="I32" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="J32" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach {{LOAN_ID}}</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="L32" s="11" t="inlineStr">
         <is>
           <t>Immediate Action: Liquidation of Pledged Mutual Fund Units due to LTV Breach SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="M32" s="11" t="inlineStr">
         <is>
           <t>LTV Breach – Liquidation of Pledged Units
 Dear {{CUSTOMER_NAME}},
@@ -3070,7 +3152,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N31" s="3" t="inlineStr">
+      <c r="N32" s="11" t="inlineStr">
         <is>
           <t>LTV Breach – Liquidation of Pledged Units
 Dear AZHAGARSAMY,
@@ -3085,74 +3167,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="O32" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="P32" s="11" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>LAMF Principal Repayment Reminder</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>The day after the loan end date (loan matured) when the outstanding principal is still not paid</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your LAMF has matured and the outstanding principal remains unpaid. You are requested to make immediate payment to avoid liquidation of MF pledged units https://lamf.shriramcredit.in/user/loans/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="I33" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="J33" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K33" s="11" t="inlineStr">
         <is>
           <t>Action Required: Principal Repayment {{LOAN_ID}}</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="L33" s="11" t="inlineStr">
         <is>
           <t>Action Required: Principal Repayment SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="M33" s="11" t="inlineStr">
         <is>
           <t>Principal Repayment for Loan Closure
 Dear {{CUSTOMER_NAME}},
@@ -3172,7 +3254,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N32" s="3" t="inlineStr">
+      <c r="N33" s="11" t="inlineStr">
         <is>
           <t>Principal Repayment for Loan Closure
 Dear AZHAGARSAMY,
@@ -3192,74 +3274,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="O33" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="P33" s="11" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>LAMF Liquidation for O/S</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>On the day the liquidation is initiated for the outstanding principal that is still unpaid after maturity</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="11" t="inlineStr">
         <is>
           <t>Dear {#alp#}, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, As the outstanding principal is still unpaid, we are initiating liquidation for recovery of outstanding dues - Shriram Credit</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="I34" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="J34" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan {{LOAN_ID}}</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="L34" s="11" t="inlineStr">
         <is>
           <t>Immediate Action: Liquidation of Pledged Mutual Fund Units for Recovery of Outstanding Loan SCCLMF20261000102</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="M34" s="11" t="inlineStr">
         <is>
           <t>Liquidation for Outstanding Loan
 Dear {{CUSTOMER_NAME}},
@@ -3274,7 +3356,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N33" s="3" t="inlineStr">
+      <c r="N34" s="11" t="inlineStr">
         <is>
           <t>Liquidation for Outstanding Loan
 Dear AZHAGARSAMY,
@@ -3289,74 +3371,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O33" s="3" t="inlineStr">
+      <c r="O34" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="P34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Foreclosure Completed</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>When the customer forecloses (pre-closes) the loan before the end of the tenure and the foreclosure is completed. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>LMS</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E35" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G35" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund account {#alphanumeric#} has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H35" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="I35" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="K35" s="13" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr">
+      <c r="L35" s="13" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation: Your Shriram Credit LAMF Has Been Closed Successfully</t>
         </is>
       </c>
-      <c r="M34" s="5" t="inlineStr">
+      <c r="M35" s="13" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation
 Dear {{CUSTOMER_NAME}},
@@ -3380,7 +3462,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N34" s="5" t="inlineStr">
+      <c r="N35" s="13" t="inlineStr">
         <is>
           <t>Loan Pre-Closure Confirmation
 Dear AZHAGARSAMY,
@@ -3404,74 +3486,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O34" s="5" t="inlineStr">
+      <c r="O35" s="13" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="P35" s="13" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Successful Loan Tenure Completion</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>When the customer completes all the EMI instalments (loan fully repaid)</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F36" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Loan fully repaid! Your MF units will be released in 2-3 working days and your loan account will be closed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="I36" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="J36" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>Congratulations on completing your loan journey</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr">
+      <c r="L36" s="11" t="inlineStr">
         <is>
           <t>Congratulations on completing your loan journey</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr">
+      <c r="M36" s="11" t="inlineStr">
         <is>
           <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
 Loan Journey Complete
@@ -3496,7 +3578,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N35" s="3" t="inlineStr">
+      <c r="N36" s="11" t="inlineStr">
         <is>
           <t>Trigger: last EMI paid (EMI type) or principal outstanding paid (Balloon type)
 Loan Journey Complete
@@ -3521,74 +3603,74 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr">
+      <c r="O36" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="P36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Loan Account Closure</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>When the loan account is closed (closed on = loan end date)</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>SMS, Mail</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your loan account {#alphanumeric#} has been successfully closed on {#alphanumeric#}. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="H37" s="11" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your loan account SCCLMF20261000102 has been successfully closed on 26-10-2027. Thank you for your association with Shriram Credit - Shriram Credit</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="I37" s="11" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr">
+      <c r="J37" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="K37" s="11" t="inlineStr">
         <is>
           <t>Your Loan Account {{LOAN_ID}} is closed successfully</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="L37" s="11" t="inlineStr">
         <is>
           <t>Your Loan Account SCCLMF20261000102 is closed successfully</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr">
+      <c r="M37" s="11" t="inlineStr">
         <is>
           <t>Trigger: manual trigger
 Attachment: NOC / Loan Closure Certificate PDF
@@ -3605,7 +3687,7 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="N36" s="3" t="inlineStr">
+      <c r="N37" s="11" t="inlineStr">
         <is>
           <t>Trigger: manual trigger
 Attachment: NOC / Loan Closure Certificate PDF
@@ -3622,87 +3704,93 @@
 © 2026 Shriram Credit Company Limited. All rights reserved.</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr">
+      <c r="O37" s="11" t="inlineStr">
         <is>
           <t>Yes
 View mail</t>
         </is>
       </c>
-      <c r="P36" s="3" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="P37" s="11" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>SMS and mail marked "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P36"/>
+  <autoFilter ref="A2:P37"/>
+  <mergeCells count="4">
+    <mergeCell ref="P1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:J1"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3715,7 +3803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3739,584 +3827,624 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="n"/>
+      <c r="M1" s="6" t="n"/>
+      <c r="N1" s="6" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Scenarios</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Sender</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Communication Type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>SMS Content Structure</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Actual SMS Content</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>SMS Header</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>SMS Available</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Mail Subject Structure</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Actual Mail Subject</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Mail Content Structure</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>Actual Mail Content</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>Mail Available</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>LAN Generated</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>When the customer clicks Continue on the Loan Application Summary page and the Loan Account Number (LAN) is generated successfully</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is {#alphanumeric#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr"/>
-      <c r="P2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="K3" s="13" t="inlineStr"/>
+      <c r="L3" s="13" t="inlineStr"/>
+      <c r="M3" s="13" t="inlineStr"/>
+      <c r="N3" s="13" t="inlineStr"/>
+      <c r="O3" s="13" t="inlineStr"/>
+      <c r="P3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>The application is still incomplete before pledging and reaches the configured expiry-reminder date (the application expires 30 days after LAN generation)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} is incomplete and will expire on {#alphanumeric#}. Please complete it before this date to avoid cancellation {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="5" t="inlineStr"/>
-      <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr"/>
-      <c r="P3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="K4" s="13" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr"/>
+      <c r="M4" s="13" t="inlineStr"/>
+      <c r="N4" s="13" t="inlineStr"/>
+      <c r="O4" s="13" t="inlineStr"/>
+      <c r="P4" s="13" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Pre-Pledge Application Discarded</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>On Day 31 the application has not been pledged or submitted, and the system discards it automatically</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="K5" s="13" t="inlineStr"/>
+      <c r="L5" s="13" t="inlineStr"/>
+      <c r="M5" s="13" t="inlineStr"/>
+      <c r="N5" s="13" t="inlineStr"/>
+      <c r="O5" s="13" t="inlineStr"/>
+      <c r="P5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Customer-Initiated Discard</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>The customer selects Discard before pledging and the application is cancelled. No backend approval – it is discarded at once</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} has been discarded as requested. You can start a new loan application anytime {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="K6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="13" t="inlineStr"/>
+      <c r="N6" s="13" t="inlineStr"/>
+      <c r="O6" s="13" t="inlineStr"/>
+      <c r="P6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Lien Marking Failed</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>When the lien marking (pledge) of the mutual fund units fails on the “Pledging of Mutual Fund” page. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="K7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr"/>
+      <c r="M7" s="13" t="inlineStr"/>
+      <c r="N7" s="13" t="inlineStr"/>
+      <c r="O7" s="13" t="inlineStr"/>
+      <c r="P7" s="13" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Post-Pledge Journey Incomplete</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Lien marking is successful, then the customer is inactive for the configured period</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Mutual Fund units are pledged for loan account {#alphanumeric#}, but your loan application is not complete yet. Please resume and complete the remaining steps {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
-      <c r="O7" s="5" t="inlineStr"/>
-      <c r="P7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="K8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="13" t="inlineStr"/>
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Post-Pledge Application Expiry Reminder</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>The application approaches its 30-day expiry date, is still not submitted and the lien is active</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your Loan Against Mutual Fund application {#alphanumeric#} will expire on {#alphanumeric#}. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date {#urg#} - Shriram Credit</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="K9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="13" t="inlineStr"/>
+      <c r="O9" s="13" t="inlineStr"/>
+      <c r="P9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Lien Removal Request Received</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>SCCL receives and records the customer’s lien removal request</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, We have received your lien removal request for loan account {#alphanumeric#}. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr"/>
-      <c r="O9" s="5" t="inlineStr"/>
-      <c r="P9" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="K10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="13" t="inlineStr"/>
+      <c r="P10" s="13" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Rows highlighted in yellow (Available = "No – to be created") are templates drafted for approval; they still have to be created and registered.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>SMS and mail marked "Not Required" are in the separate "Not Required" sheet – kept for reference only; they will not be sent.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Actual Content shows a sample with the variables filled in (sample customer AZHAGARSAMY, loan account SCCLMF20261000102).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Source: LAMF – Customer Communications page (https://azhagarvicky.github.io/SCCL-PRD/dev/lamf-journey/communications.html).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Created by Azhagarsamy Subburaj. For any observation or clarification, please reach out to azhagarsamy.s@shriramcredit.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P9"/>
+  <autoFilter ref="A2:P10"/>
+  <mergeCells count="4">
+    <mergeCell ref="P1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Communications: '-' in the Mail columns of SMS-only rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -720,11 +720,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr"/>
-      <c r="L3" s="11" t="inlineStr"/>
-      <c r="M3" s="11" t="inlineStr"/>
-      <c r="N3" s="11" t="inlineStr"/>
-      <c r="O3" s="11" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
@@ -776,11 +796,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" s="11" t="inlineStr"/>
-      <c r="L4" s="11" t="inlineStr"/>
-      <c r="M4" s="11" t="inlineStr"/>
-      <c r="N4" s="11" t="inlineStr"/>
-      <c r="O4" s="11" t="inlineStr"/>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
@@ -832,11 +872,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr"/>
-      <c r="L5" s="11" t="inlineStr"/>
-      <c r="M5" s="11" t="inlineStr"/>
-      <c r="N5" s="11" t="inlineStr"/>
-      <c r="O5" s="11" t="inlineStr"/>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1080,11 +1140,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="13" t="inlineStr"/>
-      <c r="L8" s="13" t="inlineStr"/>
-      <c r="M8" s="13" t="inlineStr"/>
-      <c r="N8" s="13" t="inlineStr"/>
-      <c r="O8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1136,11 +1216,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="13" t="inlineStr"/>
-      <c r="L9" s="13" t="inlineStr"/>
-      <c r="M9" s="13" t="inlineStr"/>
-      <c r="N9" s="13" t="inlineStr"/>
-      <c r="O9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1192,11 +1292,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K10" s="13" t="inlineStr"/>
-      <c r="L10" s="13" t="inlineStr"/>
-      <c r="M10" s="13" t="inlineStr"/>
-      <c r="N10" s="13" t="inlineStr"/>
-      <c r="O10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1248,11 +1368,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K11" s="13" t="inlineStr"/>
-      <c r="L11" s="13" t="inlineStr"/>
-      <c r="M11" s="13" t="inlineStr"/>
-      <c r="N11" s="13" t="inlineStr"/>
-      <c r="O11" s="13" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1514,11 +1654,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="11" t="inlineStr"/>
-      <c r="L14" s="11" t="inlineStr"/>
-      <c r="M14" s="11" t="inlineStr"/>
-      <c r="N14" s="11" t="inlineStr"/>
-      <c r="O14" s="11" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1669,11 +1829,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K16" s="13" t="inlineStr"/>
-      <c r="L16" s="13" t="inlineStr"/>
-      <c r="M16" s="13" t="inlineStr"/>
-      <c r="N16" s="13" t="inlineStr"/>
-      <c r="O16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P16" s="13" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1725,11 +1905,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K17" s="13" t="inlineStr"/>
-      <c r="L17" s="13" t="inlineStr"/>
-      <c r="M17" s="13" t="inlineStr"/>
-      <c r="N17" s="13" t="inlineStr"/>
-      <c r="O17" s="13" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P17" s="13" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1876,11 +2076,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr"/>
-      <c r="L19" s="11" t="inlineStr"/>
-      <c r="M19" s="11" t="inlineStr"/>
-      <c r="N19" s="11" t="inlineStr"/>
-      <c r="O19" s="11" t="inlineStr"/>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P19" s="11" t="inlineStr">
         <is>
           <t>This SMS has to come once the withdrawal OTP is verified successfully, but it currently comes only once the UTR is approved in the LMS.</t>
@@ -1936,11 +2156,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K20" s="13" t="inlineStr"/>
-      <c r="L20" s="13" t="inlineStr"/>
-      <c r="M20" s="13" t="inlineStr"/>
-      <c r="N20" s="13" t="inlineStr"/>
-      <c r="O20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
@@ -2774,11 +3014,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K28" s="11" t="inlineStr"/>
-      <c r="L28" s="11" t="inlineStr"/>
-      <c r="M28" s="11" t="inlineStr"/>
-      <c r="N28" s="11" t="inlineStr"/>
-      <c r="O28" s="11" t="inlineStr"/>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
@@ -3989,11 +4249,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr"/>
-      <c r="L3" s="13" t="inlineStr"/>
-      <c r="M3" s="13" t="inlineStr"/>
-      <c r="N3" s="13" t="inlineStr"/>
-      <c r="O3" s="13" t="inlineStr"/>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P3" s="13" t="inlineStr"/>
     </row>
     <row r="4">
@@ -4045,11 +4325,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K4" s="13" t="inlineStr"/>
-      <c r="L4" s="13" t="inlineStr"/>
-      <c r="M4" s="13" t="inlineStr"/>
-      <c r="N4" s="13" t="inlineStr"/>
-      <c r="O4" s="13" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
@@ -4101,11 +4401,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr"/>
-      <c r="L5" s="13" t="inlineStr"/>
-      <c r="M5" s="13" t="inlineStr"/>
-      <c r="N5" s="13" t="inlineStr"/>
-      <c r="O5" s="13" t="inlineStr"/>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4157,11 +4477,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K6" s="13" t="inlineStr"/>
-      <c r="L6" s="13" t="inlineStr"/>
-      <c r="M6" s="13" t="inlineStr"/>
-      <c r="N6" s="13" t="inlineStr"/>
-      <c r="O6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4213,11 +4553,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K7" s="13" t="inlineStr"/>
-      <c r="L7" s="13" t="inlineStr"/>
-      <c r="M7" s="13" t="inlineStr"/>
-      <c r="N7" s="13" t="inlineStr"/>
-      <c r="O7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4269,11 +4629,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K8" s="13" t="inlineStr"/>
-      <c r="L8" s="13" t="inlineStr"/>
-      <c r="M8" s="13" t="inlineStr"/>
-      <c r="N8" s="13" t="inlineStr"/>
-      <c r="O8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
@@ -4325,11 +4705,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K9" s="13" t="inlineStr"/>
-      <c r="L9" s="13" t="inlineStr"/>
-      <c r="M9" s="13" t="inlineStr"/>
-      <c r="N9" s="13" t="inlineStr"/>
-      <c r="O9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
@@ -4381,11 +4781,31 @@
           <t>No – to be created</t>
         </is>
       </c>
-      <c r="K10" s="13" t="inlineStr"/>
-      <c r="L10" s="13" t="inlineStr"/>
-      <c r="M10" s="13" t="inlineStr"/>
-      <c r="N10" s="13" t="inlineStr"/>
-      <c r="O10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P10" s="13" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Communications: mails drafted for rows 6-9 (to be created); Excel red mark on 'to be created' fixed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1117,7 +1117,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
@@ -1130,39 +1130,57 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has expired as it was not submitted within 30 days. Your Mutual Fund units remain lien-marked. We will share the next steps for lien removal - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="13" t="inlineStr">
+      <c r="J8" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application {{LOAN_ID}} has expired</t>
         </is>
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application SCCLMF20261000102 has expired</t>
         </is>
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Application Expired
+Dear {{CUSTOMER_NAME}},
+Your Loan Against Mutual Fund (LAMF) application {{LOAN_ID}} has expired as it was not submitted within 30 days.
+Your Mutual Fund units pledged for this application remain lien-marked. We will initiate the lien removal and keep you informed of the next steps.
+You are welcome to start a new application at any time.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Application Expired
+Dear AZHAGARSAMY,
+Your Loan Against Mutual Fund (LAMF) application SCCLMF20261000102 has expired as it was not submitted within 30 days.
+Your Mutual Fund units pledged for this application remain lien-marked. We will initiate the lien removal and keep you informed of the next steps.
+You are welcome to start a new application at any time.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P8" s="13" t="inlineStr"/>
@@ -1193,7 +1211,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1206,39 +1224,63 @@
           <t>Dear AZHAGARSAMY, Lien removal has been initiated for the Mutual Fund units pledged against loan account SCCLMF20261000102. We will update you once it is completed - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr">
+      <c r="J9" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removal initiated for your Mutual Fund units – {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removal initiated for your Mutual Fund units – SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien Removal Initiated
+Dear {{CUSTOMER_NAME}},
+We have initiated the removal of the lien on the Mutual Fund units pledged against loan account {{LOAN_ID}}.
+LIEN REMOVAL DETAILS
+Status: Lien removal initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a notification from CAMS/KFintech once your units are fully unlocked.
+We will update you once the lien removal is completed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N9" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Lien Removal Initiated
+Dear AZHAGARSAMY,
+We have initiated the removal of the lien on the Mutual Fund units pledged against loan account SCCLMF20261000102.
+LIEN REMOVAL DETAILS
+Status: Lien removal initiated
+Timeline: 2–3 working days
+Confirmation: You will receive a notification from CAMS/KFintech once your units are fully unlocked.
+We will update you once the lien removal is completed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr"/>
@@ -1269,7 +1311,7 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
@@ -1282,39 +1324,55 @@
           <t>Dear AZHAGARSAMY, The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien - Shriram Credit</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removed successfully – {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removed successfully – SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien Removal Successful
+Dear {{CUSTOMER_NAME}},
+The lien on your Mutual Fund units pledged against loan account {{LOAN_ID}} has been removed successfully. Your units are now released from lien.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Lien Removal Successful
+Dear AZHAGARSAMY,
+The lien on your Mutual Fund units pledged against loan account SCCLMF20261000102 has been removed successfully. Your units are now released from lien.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+We thank you for choosing Shriram Credit and look forward to serving you again.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P10" s="13" t="inlineStr"/>
@@ -1345,7 +1403,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -1358,39 +1416,55 @@
           <t>Dear AZHAGARSAMY, Lien removal for loan account SCCLMF20261000102 could not be completed due to a processing issue. Your Mutual Fund units remain lien-marked. We are reviewing it and will update you - Shriram Credit</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr">
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removal could not be completed – {{LOAN_ID}}</t>
         </is>
       </c>
       <c r="L11" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien removal could not be completed – SCCLMF20261000102</t>
         </is>
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Lien Removal Failed
+Dear {{CUSTOMER_NAME}},
+The removal of the lien on the Mutual Fund units pledged against loan account {{LOAN_ID}} could not be completed due to a processing issue. Your units remain lien-marked.
+Our team is reviewing it and will update you once the lien removal is completed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O11" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Lien Removal Failed
+Dear AZHAGARSAMY,
+The removal of the lien on the Mutual Fund units pledged against loan account SCCLMF20261000102 could not be completed due to a processing issue. Your units remain lien-marked.
+Our team is reviewing it and will update you once the lien removal is completed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O11" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P11" s="13" t="inlineStr"/>
@@ -1819,12 +1893,12 @@
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. Please pay the applicable charges (processing fee, lien marking and lien removal) of Rs. 92,313 using this link: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I16" s="14" t="inlineStr">
+      <c r="I16" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -1895,12 +1969,12 @@
           <t>Dear AZHAGARSAMY, We regret that your Loan Against Mutual Fund application could not be approved. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I17" s="14" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J17" s="13" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -2146,12 +2220,12 @@
           <t>Dear AZHAGARSAMY, Your withdrawal request of Rs. 10,000 for loan account SCCLMF20261000102 has been rejected. For assistance, please contact our support team - Shriram Credit</t>
         </is>
       </c>
-      <c r="I20" s="14" t="inlineStr">
+      <c r="I20" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -2596,12 +2670,12 @@
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 for loan account SCCLMF20261000102 will be presented tomorrow, 05-11-2026. Please maintain sufficient balance to avoid penal charges - Shriram Credit</t>
         </is>
       </c>
-      <c r="I24" s="14" t="inlineStr">
+      <c r="I24" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="J24" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -3678,12 +3752,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund account SCCLMF20261000102 has been foreclosed successfully. Your MF units will be released from lien in 2-3 working days - Shriram Credit</t>
         </is>
       </c>
-      <c r="I35" s="14" t="inlineStr">
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J35" s="13" t="inlineStr">
+      <c r="J35" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -3982,7 +4056,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 26 (22 available · 4 to be created) · SMS and mail: 25 · SMS only: 9 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -4239,12 +4313,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been initiated successfully. Your Loan Account Number is SCCLMF20261000102 - Shriram Credit</t>
         </is>
       </c>
-      <c r="I3" s="14" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4315,12 +4389,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 is incomplete and will expire on 26-11-2026. Please complete it before this date to avoid cancellation https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="I4" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4391,12 +4465,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 was closed as it was not completed within 30 days. We would be glad to help you - start a new application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I5" s="14" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4467,12 +4541,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 has been discarded as requested. You can start a new loan application anytime https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4543,12 +4617,12 @@
           <t>Dear AZHAGARSAMY, Lien marking of your Mutual Fund units could not be completed. Please log in and try pledging again to continue your loan application: https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr">
+      <c r="J7" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4619,12 +4693,12 @@
           <t>Dear AZHAGARSAMY, Your Mutual Fund units are pledged for loan account SCCLMF20261000102, but your loan application is not complete yet. Please resume and complete the remaining steps https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J8" s="13" t="inlineStr">
+      <c r="J8" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4695,12 +4769,12 @@
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application SCCLMF20261000102 will expire on 26-11-2026. Your Mutual Fund units are lien-marked. Please complete the remaining steps before this date https://lamf.shriramcredit.in/ - Shriram Credit</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr">
+      <c r="J9" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4771,12 +4845,12 @@
           <t>Dear AZHAGARSAMY, We have received your lien removal request for loan account SCCLMF20261000102. It is under review and we will update you once the lien removal is initiated - Shriram Credit</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>No – to be created</t>
         </is>
@@ -4818,7 +4892,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 22 (22 available) · SMS and mail: 21 · SMS only: 13 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 26 (22 available · 4 to be created) · SMS and mail: 25 · SMS only: 9 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: mail drafted for row 12 LAMF Application Submit (to be created)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1680,80 +1680,98 @@
       <c r="P13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>LAMF Application Submit</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Once the E-Mandate is completed successfully – the loan application is then considered submitted</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>SMS, Mail</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Dear {#alp#}, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your Loan Against Mutual Fund application has been successfully submitted - Shriram Credit</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="I14" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="J14" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" s="11" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>Your LAMF application {{LOAN_ID}} has been submitted successfully</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Your LAMF application SCCLMF20261000102 has been submitted successfully</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>Application Submitted
+Dear {{CUSTOMER_NAME}},
+Thank you for completing the E-Mandate. Your Loan Against Mutual Fund (LAMF) application {{LOAN_ID}} has been submitted successfully.
+Our team will now review your application, and you will be notified once your loan account is opened.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>Application Submitted
+Dear AZHAGARSAMY,
+Thank you for completing the E-Mandate. Your Loan Against Mutual Fund (LAMF) application SCCLMF20261000102 has been submitted successfully.
+Our team will now review your application, and you will be notified once your loan account is opened.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Thank you for choosing Shriram Credit as your trusted financial partner. We look forward to supporting you throughout your loan journey.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O14" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="P14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -4056,7 +4074,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 26 (22 available · 4 to be created) · SMS and mail: 25 · SMS only: 9 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 27 (22 available · 5 to be created) · SMS and mail: 26 · SMS only: 8 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4910,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 26 (22 available · 4 to be created) · SMS and mail: 25 · SMS only: 9 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 27 (22 available · 5 to be created) · SMS and mail: 26 · SMS only: 8 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: mails drafted for rows 14 and 15 (rejection with / without payment link)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1898,7 +1898,7 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
@@ -1923,27 +1923,51 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application {{LOAN_ID}} could not be approved</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application SCCLMF20261000102 could not be approved</t>
         </is>
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Application Not Approved
+Dear {{CUSTOMER_NAME}},
+We regret to inform you that your Loan Against Mutual Fund (LAMF) application {{LOAN_ID}} could not be approved after our review.
+CHARGES PAYABLE
+Processing fee, lien marking and lien removal charges: ₹{{CHARGES_AMOUNT}}
+Please pay the applicable charges using the link below.
+[Make Payment →] ({{PAYMENT_LINK}})
+Once the payment is received, the lien on your Mutual Fund units will be removed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N16" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O16" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Application Not Approved
+Dear AZHAGARSAMY,
+We regret to inform you that your Loan Against Mutual Fund (LAMF) application SCCLMF20261000102 could not be approved after our review.
+CHARGES PAYABLE
+Processing fee, lien marking and lien removal charges: ₹92,313
+Please pay the applicable charges using the link below.
+[Make Payment →] (https://lamf.shriramcredit.in/)
+Once the payment is received, the lien on your Mutual Fund units will be removed.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O16" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P16" s="13" t="inlineStr"/>
@@ -1974,7 +1998,7 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
@@ -1999,27 +2023,43 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application {{LOAN_ID}} could not be approved</t>
         </is>
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your LAMF application SCCLMF20261000102 could not be approved</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Application Not Approved
+Dear {{CUSTOMER_NAME}},
+We regret to inform you that your Loan Against Mutual Fund (LAMF) application {{LOAN_ID}} could not be approved after our review.
+There are no charges payable by you for this application.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N17" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Application Not Approved
+Dear AZHAGARSAMY,
+We regret to inform you that your Loan Against Mutual Fund (LAMF) application SCCLMF20261000102 could not be approved after our review.
+There are no charges payable by you for this application.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O17" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P17" s="13" t="inlineStr"/>
@@ -4074,7 +4114,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 27 (22 available · 5 to be created) · SMS and mail: 26 · SMS only: 8 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 29 (22 available · 7 to be created) · SMS and mail: 28 · SMS only: 6 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4950,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 27 (22 available · 5 to be created) · SMS and mail: 26 · SMS only: 8 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 29 (22 available · 7 to be created) · SMS and mail: 28 · SMS only: 6 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: rows 14/15 scenarios – LMS options Rejected with / without Charges
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITH payment link, when the customer has charges to pay (processing fee, lien marking and lien removal). Template drafted by Claude for approval; to be created and registered</t>
+          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS with the option “Rejected with Charges” – the customer has to pay the charges (processing fee, lien marking and lien removal), so the communication carries the payment link. One common communication for either rejection. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS – one common SMS for either rejection – WITHOUT payment link, when there are no charges for the customer to pay. Template drafted by Claude for approval; to be created and registered</t>
+          <t>When the OPS team rejects the Loan Account Opening or the Loan Lodgement in the backend LMS with the option “Rejected without Charges” – the charges are waived for the customer (e.g. an internal employee who completed a testing scenario), so the communication has no payment link. One common communication for either rejection. Template drafted by Claude for approval; to be created and registered</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -2036,7 +2036,7 @@
           <t>Application Not Approved
 Dear {{CUSTOMER_NAME}},
 We regret to inform you that your Loan Against Mutual Fund (LAMF) application {{LOAN_ID}} could not be approved after our review.
-There are no charges payable by you for this application.
+The applicable charges for this application have been waived, so no payment is required from you.
 Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
 Warm regards,
 Team Shriram Credit
@@ -2049,7 +2049,7 @@
           <t>Application Not Approved
 Dear AZHAGARSAMY,
 We regret to inform you that your Loan Against Mutual Fund (LAMF) application SCCLMF20261000102 could not be approved after our review.
-There are no charges payable by you for this application.
+The applicable charges for this application have been waived, so no payment is required from you.
 Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
 Warm regards,
 Team Shriram Credit

</xml_diff>

<commit_message>
Communications: mail drafted for row 18 Withdrawal Rejected (to be created)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>SMS, Mail</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
@@ -2290,27 +2290,53 @@
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your withdrawal request for loan account {{LOAN_ID}} has been rejected</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Your withdrawal request for loan account SCCLMF20261000102 has been rejected</t>
         </is>
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Withdrawal Request Rejected
+Dear {{CUSTOMER_NAME}},
+We regret to inform you that your withdrawal request of ₹{{WITHDRAWAL_AMOUNT}} for loan account {{LOAN_ID}} has been rejected after our review. No amount has been disbursed against this request.
+WITHDRAWAL DETAILS
+Loan Account ID: {{LOAN_ID}}
+Withdrawal Amount: ₹{{WITHDRAWAL_AMOUNT}}
+Request Date: {{REQUEST_DATE}}
+Status: Rejected
+You may place a new withdrawal request at any time, subject to your available balance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
         </is>
       </c>
       <c r="N20" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O20" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>Withdrawal Request Rejected
+Dear AZHAGARSAMY,
+We regret to inform you that your withdrawal request of ₹10,000 for loan account SCCLMF20261000102 has been rejected after our review. No amount has been disbursed against this request.
+WITHDRAWAL DETAILS
+Loan Account ID: SCCLMF20261000102
+Withdrawal Amount: ₹10,000
+Request Date: 02-11-2026
+Status: Rejected
+You may place a new withdrawal request at any time, subject to your available balance.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr"/>
@@ -4114,7 +4140,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 29 (22 available · 7 to be created) · SMS and mail: 28 · SMS only: 6 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 30 (22 available · 8 to be created) · SMS and mail: 29 · SMS only: 5 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4976,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 29 (22 available · 7 to be created) · SMS and mail: 28 · SMS only: 6 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 30 (22 available · 8 to be created) · SMS and mail: 29 · SMS only: 5 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: mail drafted for row 26 EMI Resubmission Success (to be created)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -3124,80 +3124,106 @@
       <c r="P27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n">
+      <c r="A28" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>EMI Resubmission Success</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>Notifying the customer when the EMI resubmission is successful</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="inlineStr">
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>SMS, Mail</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your EMI of Rs. {#alphanumeric#} was successfully debited on {#alphanumeric#}. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H28" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your EMI of Rs. 10,000 was successfully debited on 10-11-2026. Thank you for your payment - Shriram Credit</t>
         </is>
       </c>
-      <c r="I28" s="11" t="inlineStr">
+      <c r="I28" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J28" s="11" t="inlineStr">
+      <c r="J28" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P28" s="11" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>Your re-presented EMI of ₹{{EMI_AMOUNT}} has been successfully deducted</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Your re-presented EMI of ₹10,000 has been successfully deducted</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t>EMI Payment Confirmed
+Dear {{CUSTOMER_NAME}},
+We are writing to confirm that your EMI of ₹{{EMI_AMOUNT}} for the loan account {{LOAN_ID}}, which was re-presented after the earlier failed attempt, was successfully debited on {{DEDUCTION_DATE}} from your registered bank account.
+EMI DETAILS
+Loan Account Number: {{LOAN_ID}}
+EMI Amount: ₹{{EMI_AMOUNT}}
+Deduction Date: {{DEDUCTION_DATE}}
+Next EMI Due Date: {{NEXT_EMI_DATE}}
+Thank you for your payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="inlineStr">
+        <is>
+          <t>EMI Payment Confirmed
+Dear AZHAGARSAMY,
+We are writing to confirm that your EMI of ₹10,000 for the loan account SCCLMF20261000102, which was re-presented after the earlier failed attempt, was successfully debited on 10-11-2026 from your registered bank account.
+EMI DETAILS
+Loan Account Number: SCCLMF20261000102
+EMI Amount: ₹10,000
+Deduction Date: 10-11-2026
+Next EMI Due Date: 05-12-2026
+Thank you for your payment. Regular EMI payments help maintain a strong credit history and a smooth loan journey.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O28" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="P28" s="13" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -4140,7 +4166,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 30 (22 available · 8 to be created) · SMS and mail: 29 · SMS only: 5 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 31 (22 available · 9 to be created) · SMS and mail: 30 · SMS only: 4 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -4976,7 +5002,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 30 (22 available · 8 to be created) · SMS and mail: 29 · SMS only: 5 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 31 (22 available · 9 to be created) · SMS and mail: 30 · SMS only: 4 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Communications: View link for row 19 (first disbursement mail built as HTML from the shared text)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2478,7 +2478,8 @@
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes
+View mail</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
@@ -4220,21 +4221,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Communications: mail drafted for row 17 Withdrawal confirmed (to be created)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsVs5RNJ4JXhPDXV9bN1Kw
</commit_message>
<xml_diff>
--- a/exports/LAMF_Customer_Communications.xlsx
+++ b/exports/LAMF_Customer_Communications.xlsx
@@ -2160,80 +2160,108 @@
       <c r="P18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>On the completion of each withdrawal by the customer (withdrawal request confirmed)</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>LOS</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>SCCL</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>SMS, Mail</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
         <is>
           <t>Dear {#alphanumeric#}, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>Dear AZHAGARSAMY, Your withdrawal request is confirmed. Your loan amount will be disbursed to your bank account shortly - Shriram Credit</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr">
         <is>
           <t>SGRCDT-T</t>
         </is>
       </c>
-      <c r="J19" s="11" t="inlineStr">
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N19" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P19" s="11" t="inlineStr">
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>Your withdrawal request for loan account {{LOAN_ID}} is confirmed</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>Your withdrawal request for loan account SCCLMF20261000102 is confirmed</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawal Request Confirmed
+Dear {{CUSTOMER_NAME}},
+Your withdrawal request of ₹{{WITHDRAWAL_AMOUNT}} for loan account {{LOAN_ID}} has been confirmed. The amount will be disbursed to your registered bank account shortly.
+WITHDRAWAL DETAILS
+Loan Account ID: {{LOAN_ID}}
+Withdrawal Amount: ₹{{WITHDRAWAL_AMOUNT}}
+Request Date: {{REQUEST_DATE}}
+Bank Account Number: {{BANK_ACCOUNT_NUMBER}}
+Status: Confirmed
+You will receive a separate confirmation once the amount is credited to your bank account.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawal Request Confirmed
+Dear AZHAGARSAMY,
+Your withdrawal request of ₹10,000 for loan account SCCLMF20261000102 has been confirmed. The amount will be disbursed to your registered bank account shortly.
+WITHDRAWAL DETAILS
+Loan Account ID: SCCLMF20261000102
+Withdrawal Amount: ₹10,000
+Request Date: 02-11-2026
+Bank Account Number: XXXXXXXX8736
+Status: Confirmed
+You will receive a separate confirmation once the amount is credited to your bank account.
+Should you have any questions, require clarification, or assistance, please feel free to reach out to our customer support at lassupport@shriramcredit.in. Our team will be happy to assist you.
+Warm regards,
+Team Shriram Credit
+Disclaimer:
+This is an automated reminder. Please do not reply to this message, as the mailbox is not monitored and you will not receive a response. Loan against Securities is for personal use only and cannot be used for speculative activities, capital market-related purposes, or anti-social purposes.</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>No – to be created</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
         <is>
           <t>This SMS has to come once the withdrawal OTP is verified successfully, but it currently comes only once the UTR is approved in the LMS.</t>
         </is>
@@ -4167,7 +4195,7 @@
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 31 (22 available · 9 to be created) · SMS and mail: 30 · SMS only: 4 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 32 (22 available · 10 to be created) · SMS and mail: 31 · SMS only: 3 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5032,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 31 (22 available · 9 to be created) · SMS and mail: 30 · SMS only: 4 · Mail only: 1 · Not required: 8 (separate table below)</t>
+          <t>Summary – Total scenarios: 35 · SMS: 34 (25 available · 9 to be created) · Mail: 32 (22 available · 10 to be created) · SMS and mail: 31 · SMS only: 3 · Mail only: 1 · Not required: 8 (separate table below)</t>
         </is>
       </c>
     </row>

</xml_diff>